<commit_message>
🔒 [FULL] Daily chip data 2026-10-02 04:01
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-10.xlsx
+++ b/data/reports/chip_radar_2026-10.xlsx
@@ -21,7 +21,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="14">
+  <numFmts count="15">
     <numFmt numFmtId="164" formatCode="0%&quot; (13/13 ・昨100/5d100)&quot;"/>
     <numFmt numFmtId="165" formatCode="+0&quot; 億 (昨-42/5d-70)&quot;;-0&quot; 億 (昨-42/5d-70)&quot;;0&quot; 億&quot;"/>
     <numFmt numFmtId="166" formatCode="0&quot; 檔 +11億 &quot;&quot;(昨7/5d12)&quot;"/>
@@ -36,6 +36,7 @@
     <numFmt numFmtId="175" formatCode="0&quot;%&quot;"/>
     <numFmt numFmtId="176" formatCode="#,##0.00;-#,##0.00"/>
     <numFmt numFmtId="177" formatCode="&quot;📅 明日預測 ↕ 中性 &quot;0.0&quot;% 信心 — P/C Ratio 主推 — 3 檔焦點&quot;"/>
+    <numFmt numFmtId="178" formatCode="0.0%&quot; 市-760億 &quot;&quot;(昨16/5d18)&quot;"/>
   </numFmts>
   <fonts count="52">
     <font>
@@ -600,7 +601,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="235">
+  <cellXfs count="236">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1138,6 +1139,9 @@
     <xf numFmtId="176" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="178" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1223,9 +1227,9 @@
     <comment ref="D18" authorId="0" shapeId="0">
       <text>
         <t>⚠️ 假共識警示
-領頭大戶「陳律師」獨佔比 57.2%
+領頭大戶「陳律師」獨佔比 56.8%
   • 領頭金額 15,983 萬
-  • 合計淨買 27,965 萬
+  • 合計淨買 28,161 萬
   • 大戶數 13 位 (名義共識)
 判讀: 名義 13 位大戶共識,
 實質 1 人下注佔 57%,
@@ -1736,7 +1740,7 @@
         <v>12</v>
       </c>
       <c r="F16" s="15" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G16" s="16" t="inlineStr">
         <is>
@@ -1752,7 +1756,7 @@
         </is>
       </c>
       <c r="J16" s="18" t="n">
-        <v>5367</v>
+        <v>4797</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
@@ -1766,7 +1770,7 @@
         <v>9</v>
       </c>
       <c r="N16" s="17" t="n">
-        <v>32785</v>
+        <v>32215</v>
       </c>
     </row>
     <row r="17">
@@ -1817,7 +1821,7 @@
         <v>9</v>
       </c>
       <c r="N17" s="17" t="n">
-        <v>32558</v>
+        <v>32141</v>
       </c>
     </row>
     <row r="18">
@@ -1838,7 +1842,7 @@
         <v>13</v>
       </c>
       <c r="F18" s="15" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G18" s="16" t="inlineStr">
         <is>
@@ -1868,7 +1872,7 @@
         <v>10</v>
       </c>
       <c r="N18" s="17" t="n">
-        <v>27966</v>
+        <v>28161</v>
       </c>
     </row>
     <row r="19">
@@ -1886,10 +1890,10 @@
         </is>
       </c>
       <c r="E19" s="14" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F19" s="15" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G19" s="16" t="inlineStr">
         <is>
@@ -1916,10 +1920,10 @@
         <v>784</v>
       </c>
       <c r="M19" s="19" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N19" s="17" t="n">
-        <v>7102</v>
+        <v>6990</v>
       </c>
     </row>
     <row r="20">
@@ -1995,7 +1999,7 @@
         </is>
       </c>
       <c r="G23" s="208" t="n">
-        <v>-111.19233</v>
+        <v>-112.8181</v>
       </c>
     </row>
     <row r="24" ht="28" customHeight="1">
@@ -2012,8 +2016,8 @@
           <t>Q4 追蹤佔比</t>
         </is>
       </c>
-      <c r="G24" s="210" t="n">
-        <v>0.200330980029177</v>
+      <c r="G24" s="235" t="n">
+        <v>0.1999189844850497</v>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">
@@ -2124,11 +2128,11 @@
         </is>
       </c>
       <c r="D31" s="34" t="n">
-        <v>1262925</v>
+        <v>1254658</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>25.7%</t>
+          <t>25.6%</t>
         </is>
       </c>
       <c r="F31" t="n">
@@ -2192,7 +2196,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>9.6%</t>
+          <t>9.7%</t>
         </is>
       </c>
       <c r="F33" t="n">
@@ -2338,7 +2342,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>陳族元</t>
+          <t>Tradow</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2348,12 +2352,12 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>陳族元 今日買進 9 檔新標的 (過去從沒買過)</t>
+          <t>Tradow 今日買進 7 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>9 檔</t>
+          <t>7 檔</t>
         </is>
       </c>
     </row>
@@ -2365,7 +2369,7 @@
       </c>
       <c r="C42" s="41" t="inlineStr">
         <is>
-          <t>Tradow</t>
+          <t>大牌分析師</t>
         </is>
       </c>
       <c r="D42" s="41" t="inlineStr">
@@ -2375,7 +2379,7 @@
       </c>
       <c r="E42" s="41" t="inlineStr">
         <is>
-          <t>Tradow 今日買進 7 檔新標的 (過去從沒買過)</t>
+          <t>大牌分析師 今日買進 7 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F42" s="41" t="inlineStr">
@@ -2392,7 +2396,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>大牌分析師</t>
+          <t>巨人傑</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -2402,7 +2406,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>大牌分析師 今日買進 7 檔新標的 (過去從沒買過)</t>
+          <t>巨人傑 今日買進 7 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2419,7 +2423,7 @@
       </c>
       <c r="C44" s="41" t="inlineStr">
         <is>
-          <t>巨人傑</t>
+          <t>布哥/n_nchang</t>
         </is>
       </c>
       <c r="D44" s="41" t="inlineStr">
@@ -2429,7 +2433,7 @@
       </c>
       <c r="E44" s="41" t="inlineStr">
         <is>
-          <t>巨人傑 今日買進 7 檔新標的 (過去從沒買過)</t>
+          <t>布哥/n_nchang 今日買進 7 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F44" s="41" t="inlineStr">
@@ -2446,7 +2450,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>布哥/n_nchang</t>
+          <t>蔣承翰</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -2456,7 +2460,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>布哥/n_nchang 今日買進 7 檔新標的 (過去從沒買過)</t>
+          <t>蔣承翰 今日買進 7 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2473,7 +2477,7 @@
       </c>
       <c r="C46" s="41" t="inlineStr">
         <is>
-          <t>蔣承翰</t>
+          <t>民哥</t>
         </is>
       </c>
       <c r="D46" s="41" t="inlineStr">
@@ -2483,12 +2487,12 @@
       </c>
       <c r="E46" s="41" t="inlineStr">
         <is>
-          <t>蔣承翰 今日買進 7 檔新標的 (過去從沒買過)</t>
+          <t>民哥 今日買進 6 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F46" s="41" t="inlineStr">
         <is>
-          <t>7 檔</t>
+          <t>6 檔</t>
         </is>
       </c>
     </row>
@@ -2500,7 +2504,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>民哥</t>
+          <t>陳族元</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2510,7 +2514,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>民哥 今日買進 6 檔新標的 (過去從沒買過)</t>
+          <t>陳族元 今日買進 6 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2827,7 +2831,7 @@
         </is>
       </c>
       <c r="C63" s="34" t="n">
-        <v>1184180</v>
+        <v>1175960</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
@@ -2854,7 +2858,7 @@
         <v>60746</v>
       </c>
       <c r="J63" s="213" t="n">
-        <v>0.3783509149746875</v>
+        <v>0.380995632335176</v>
       </c>
     </row>
     <row r="64">
@@ -4248,7 +4252,7 @@
     <row r="11">
       <c r="C11" s="73" t="inlineStr">
         <is>
-          <t>④ 台新新光金 (2887) · 11 大戶</t>
+          <t>④ 台新新光金 (2887) · 10 大戶</t>
         </is>
       </c>
     </row>
@@ -4346,7 +4350,7 @@
     <row r="29" ht="22" customHeight="1">
       <c r="C29" s="77" t="inlineStr">
         <is>
-          <t>-111 億 淨買</t>
+          <t>-113 億 淨買</t>
         </is>
       </c>
     </row>
@@ -14925,29 +14929,29 @@
       <c r="C191" s="141" t="n"/>
       <c r="D191" s="138" t="inlineStr">
         <is>
-          <t>環球晶(6488)</t>
+          <t>友達(2409)</t>
         </is>
       </c>
       <c r="E191" s="139" t="n">
-        <v>33</v>
+        <v>966</v>
       </c>
       <c r="F191" s="139" t="n">
-        <v>27</v>
+        <v>890</v>
       </c>
       <c r="G191" s="139" t="n">
-        <v>3552</v>
+        <v>3700</v>
       </c>
       <c r="H191" s="139" t="n">
-        <v>2943</v>
+        <v>3409</v>
       </c>
       <c r="I191" s="139" t="n">
-        <v>609</v>
+        <v>291</v>
       </c>
       <c r="J191" s="140" t="n">
-        <v>1076.42</v>
+        <v>38.3</v>
       </c>
       <c r="K191" s="140" t="n">
-        <v>1090</v>
+        <v>38.3</v>
       </c>
       <c r="L191" s="232">
         <f>F191*(K191-J191)</f>
@@ -14960,31 +14964,31 @@
       <c r="C192" s="141" t="n"/>
       <c r="D192" s="138" t="inlineStr">
         <is>
-          <t>亞翔(6139)</t>
+          <t>環球晶(6488)</t>
         </is>
       </c>
       <c r="E192" s="139" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F192" s="139" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="G192" s="139" t="n">
-        <v>2590</v>
+        <v>3552</v>
       </c>
       <c r="H192" s="139" t="n">
-        <v>1822</v>
+        <v>2943</v>
       </c>
       <c r="I192" s="139" t="n">
-        <v>768</v>
+        <v>609</v>
       </c>
       <c r="J192" s="140" t="n">
-        <v>761.8200000000001</v>
+        <v>1076.42</v>
       </c>
       <c r="K192" s="140" t="n">
-        <v>759.29</v>
-      </c>
-      <c r="L192" s="233">
+        <v>1090</v>
+      </c>
+      <c r="L192" s="232">
         <f>F192*(K192-J192)</f>
         <v/>
       </c>
@@ -14995,31 +14999,31 @@
       <c r="C193" s="141" t="n"/>
       <c r="D193" s="138" t="inlineStr">
         <is>
-          <t>合晶(6182)</t>
+          <t>亞翔(6139)</t>
         </is>
       </c>
       <c r="E193" s="139" t="n">
-        <v>198</v>
+        <v>34</v>
       </c>
       <c r="F193" s="139" t="n">
-        <v>148</v>
+        <v>24</v>
       </c>
       <c r="G193" s="139" t="n">
-        <v>2574</v>
+        <v>2590</v>
       </c>
       <c r="H193" s="139" t="n">
-        <v>1924</v>
+        <v>1822</v>
       </c>
       <c r="I193" s="139" t="n">
-        <v>650</v>
+        <v>768</v>
       </c>
       <c r="J193" s="140" t="n">
-        <v>130</v>
+        <v>761.8200000000001</v>
       </c>
       <c r="K193" s="140" t="n">
-        <v>130</v>
-      </c>
-      <c r="L193" s="232">
+        <v>759.29</v>
+      </c>
+      <c r="L193" s="233">
         <f>F193*(K193-J193)</f>
         <v/>
       </c>
@@ -15030,29 +15034,29 @@
       <c r="C194" s="141" t="n"/>
       <c r="D194" s="138" t="inlineStr">
         <is>
-          <t>禾伸堂(3026)</t>
+          <t>聯發科(2454)</t>
         </is>
       </c>
       <c r="E194" s="139" t="n">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="F194" s="139" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="G194" s="139" t="n">
-        <v>2471</v>
+        <v>2238</v>
       </c>
       <c r="H194" s="139" t="n">
-        <v>682</v>
+        <v>1162</v>
       </c>
       <c r="I194" s="139" t="n">
-        <v>1789</v>
+        <v>1076</v>
       </c>
       <c r="J194" s="140" t="n">
-        <v>852</v>
+        <v>5593.75</v>
       </c>
       <c r="K194" s="140" t="n">
-        <v>852</v>
+        <v>5810.5</v>
       </c>
       <c r="L194" s="232">
         <f>F194*(K194-J194)</f>
@@ -15065,29 +15069,29 @@
       <c r="C195" s="141" t="n"/>
       <c r="D195" s="138" t="inlineStr">
         <is>
-          <t>群創(3481)</t>
+          <t>頎邦(6147)</t>
         </is>
       </c>
       <c r="E195" s="139" t="n">
-        <v>440</v>
+        <v>94</v>
       </c>
       <c r="F195" s="139" t="n">
-        <v>331</v>
+        <v>53</v>
       </c>
       <c r="G195" s="139" t="n">
-        <v>2301</v>
+        <v>2084</v>
       </c>
       <c r="H195" s="139" t="n">
-        <v>1731</v>
+        <v>1194</v>
       </c>
       <c r="I195" s="139" t="n">
-        <v>570</v>
+        <v>890</v>
       </c>
       <c r="J195" s="140" t="n">
-        <v>52.3</v>
+        <v>221.71</v>
       </c>
       <c r="K195" s="140" t="n">
-        <v>52.3</v>
+        <v>225.28</v>
       </c>
       <c r="L195" s="232">
         <f>F195*(K195-J195)</f>
@@ -15100,31 +15104,31 @@
       <c r="C196" s="141" t="n"/>
       <c r="D196" s="138" t="inlineStr">
         <is>
-          <t>聯發科(2454)</t>
+          <t>旺矽(6223)</t>
         </is>
       </c>
       <c r="E196" s="139" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F196" s="139" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G196" s="139" t="n">
-        <v>2238</v>
+        <v>1681</v>
       </c>
       <c r="H196" s="139" t="n">
-        <v>1162</v>
+        <v>58</v>
       </c>
       <c r="I196" s="139" t="n">
-        <v>1076</v>
+        <v>1623</v>
       </c>
       <c r="J196" s="140" t="n">
-        <v>5593.75</v>
+        <v>5604</v>
       </c>
       <c r="K196" s="140" t="n">
-        <v>5810.5</v>
-      </c>
-      <c r="L196" s="232">
+        <v>583</v>
+      </c>
+      <c r="L196" s="233">
         <f>F196*(K196-J196)</f>
         <v/>
       </c>
@@ -15135,29 +15139,29 @@
       <c r="C197" s="141" t="n"/>
       <c r="D197" s="138" t="inlineStr">
         <is>
-          <t>友達(2409)</t>
+          <t>台達電(2308)</t>
         </is>
       </c>
       <c r="E197" s="139" t="n">
-        <v>561</v>
+        <v>9</v>
       </c>
       <c r="F197" s="139" t="n">
-        <v>376</v>
+        <v>5</v>
       </c>
       <c r="G197" s="139" t="n">
-        <v>2149</v>
+        <v>1674</v>
       </c>
       <c r="H197" s="139" t="n">
-        <v>1440</v>
+        <v>1048</v>
       </c>
       <c r="I197" s="139" t="n">
-        <v>709</v>
+        <v>626</v>
       </c>
       <c r="J197" s="140" t="n">
-        <v>38.3</v>
+        <v>1860.56</v>
       </c>
       <c r="K197" s="140" t="n">
-        <v>38.3</v>
+        <v>2095.4</v>
       </c>
       <c r="L197" s="232">
         <f>F197*(K197-J197)</f>
@@ -15170,29 +15174,29 @@
       <c r="C198" s="141" t="n"/>
       <c r="D198" s="138" t="inlineStr">
         <is>
-          <t>頎邦(6147)</t>
+          <t>藥華藥(6446)</t>
         </is>
       </c>
       <c r="E198" s="139" t="n">
-        <v>92</v>
+        <v>14</v>
       </c>
       <c r="F198" s="139" t="n">
-        <v>53</v>
+        <v>1</v>
       </c>
       <c r="G198" s="139" t="n">
-        <v>2084</v>
+        <v>1671</v>
       </c>
       <c r="H198" s="139" t="n">
-        <v>1194</v>
+        <v>5</v>
       </c>
       <c r="I198" s="139" t="n">
-        <v>890</v>
+        <v>1666</v>
       </c>
       <c r="J198" s="140" t="n">
-        <v>226.53</v>
+        <v>1193.64</v>
       </c>
       <c r="K198" s="140" t="n">
-        <v>225.28</v>
+        <v>47</v>
       </c>
       <c r="L198" s="233">
         <f>F198*(K198-J198)</f>
@@ -15205,29 +15209,29 @@
       <c r="C199" s="141" t="n"/>
       <c r="D199" s="138" t="inlineStr">
         <is>
-          <t>旺矽(6223)</t>
+          <t>彩晶(6116)</t>
         </is>
       </c>
       <c r="E199" s="139" t="n">
-        <v>3</v>
+        <v>934</v>
       </c>
       <c r="F199" s="139" t="n">
-        <v>1</v>
+        <v>61</v>
       </c>
       <c r="G199" s="139" t="n">
-        <v>1681</v>
+        <v>1508</v>
       </c>
       <c r="H199" s="139" t="n">
-        <v>58</v>
+        <v>97</v>
       </c>
       <c r="I199" s="139" t="n">
-        <v>1623</v>
+        <v>1411</v>
       </c>
       <c r="J199" s="140" t="n">
-        <v>5604</v>
+        <v>16.14</v>
       </c>
       <c r="K199" s="140" t="n">
-        <v>583</v>
+        <v>15.97</v>
       </c>
       <c r="L199" s="233">
         <f>F199*(K199-J199)</f>
@@ -25710,7 +25714,7 @@
     <row r="485" ht="16.5" customHeight="1">
       <c r="A485" s="205" t="inlineStr">
         <is>
-          <t>ⓘ histock top-buyer 資料 fetched @ 2026-10-01 19:09 | 0/12 success</t>
+          <t>ⓘ histock top-buyer 資料 fetched @ 2026-10-01 20:01 | 0/12 success</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-10-02 04:46
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-10.xlsx
+++ b/data/reports/chip_radar_2026-10.xlsx
@@ -21,7 +21,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="15">
+  <numFmts count="16">
     <numFmt numFmtId="164" formatCode="0%&quot; (13/13 ・昨100/5d100)&quot;"/>
     <numFmt numFmtId="165" formatCode="+0&quot; 億 (昨-42/5d-70)&quot;;-0&quot; 億 (昨-42/5d-70)&quot;;0&quot; 億&quot;"/>
     <numFmt numFmtId="166" formatCode="0&quot; 檔 +11億 &quot;&quot;(昨7/5d12)&quot;"/>
@@ -37,6 +37,7 @@
     <numFmt numFmtId="176" formatCode="#,##0.00;-#,##0.00"/>
     <numFmt numFmtId="177" formatCode="&quot;📅 明日預測 ↕ 中性 &quot;0.0&quot;% 信心 — P/C Ratio 主推 — 3 檔焦點&quot;"/>
     <numFmt numFmtId="178" formatCode="0.0%&quot; 市-760億 &quot;&quot;(昨16/5d18)&quot;"/>
+    <numFmt numFmtId="179" formatCode="0.0%&quot; 市-758億 &quot;&quot;(昨16/5d18)&quot;"/>
   </numFmts>
   <fonts count="52">
     <font>
@@ -601,7 +602,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="236">
+  <cellXfs count="237">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1142,6 +1143,9 @@
     <xf numFmtId="178" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="179" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1588,7 +1592,7 @@
     <row r="4" ht="22" customHeight="1">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>💡 📌 一般共識 3481 / 2409 / 2883 (Q5 中性, 中性信號)  |  避開 — 除權息 2 檔: 2323, 9927 | 明日恐處置 3 檔: 3625/4304/4971  |  訊號: 中性但 hot 多 (20 個信號 — 留意)</t>
+          <t>💡 📌 一般共識 3481 / 2409 / 2883 (Q5 中性, 中性信號)  |  避開 — 明日恐處置 3 檔: 3625/4304/4971  |  訊號: 中性但 hot 多 (20 個信號 — 留意)</t>
         </is>
       </c>
     </row>
@@ -1740,7 +1744,7 @@
         <v>12</v>
       </c>
       <c r="F16" s="15" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G16" s="16" t="inlineStr">
         <is>
@@ -1756,7 +1760,7 @@
         </is>
       </c>
       <c r="J16" s="18" t="n">
-        <v>4797</v>
+        <v>5401</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
@@ -1770,7 +1774,7 @@
         <v>9</v>
       </c>
       <c r="N16" s="17" t="n">
-        <v>32215</v>
+        <v>32819</v>
       </c>
     </row>
     <row r="17">
@@ -1821,7 +1825,7 @@
         <v>9</v>
       </c>
       <c r="N17" s="17" t="n">
-        <v>32141</v>
+        <v>32572</v>
       </c>
     </row>
     <row r="18">
@@ -1999,7 +2003,7 @@
         </is>
       </c>
       <c r="G23" s="208" t="n">
-        <v>-112.8181</v>
+        <v>-111.41686</v>
       </c>
     </row>
     <row r="24" ht="28" customHeight="1">
@@ -2016,8 +2020,8 @@
           <t>Q4 追蹤佔比</t>
         </is>
       </c>
-      <c r="G24" s="235" t="n">
-        <v>0.1999189844850497</v>
+      <c r="G24" s="236" t="n">
+        <v>0.1998182239225885</v>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">
@@ -2128,11 +2132,11 @@
         </is>
       </c>
       <c r="D31" s="34" t="n">
-        <v>1254658</v>
+        <v>1251568</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>25.6%</t>
+          <t>25.5%</t>
         </is>
       </c>
       <c r="F31" t="n">
@@ -2176,7 +2180,7 @@
         </is>
       </c>
       <c r="H32" s="34" t="n">
-        <v>182044</v>
+        <v>181434</v>
       </c>
       <c r="I32" s="212" t="n">
         <v>0.0483</v>
@@ -2240,7 +2244,7 @@
         </is>
       </c>
       <c r="H34" s="34" t="n">
-        <v>95540</v>
+        <v>95565</v>
       </c>
       <c r="I34" s="212" t="n">
         <v>0.0453</v>
@@ -2504,7 +2508,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>陳族元</t>
+          <t>竹科主力分點</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2514,12 +2518,12 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>陳族元 今日買進 6 檔新標的 (過去從沒買過)</t>
+          <t>竹科主力分點 今日買進 5 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>6 檔</t>
+          <t>5 檔</t>
         </is>
       </c>
     </row>
@@ -2531,7 +2535,7 @@
       </c>
       <c r="C48" s="41" t="inlineStr">
         <is>
-          <t>竹科主力分點</t>
+          <t>陳律師</t>
         </is>
       </c>
       <c r="D48" s="41" t="inlineStr">
@@ -2541,7 +2545,7 @@
       </c>
       <c r="E48" s="41" t="inlineStr">
         <is>
-          <t>竹科主力分點 今日買進 5 檔新標的 (過去從沒買過)</t>
+          <t>陳律師 今日買進 5 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F48" s="41" t="inlineStr">
@@ -2633,11 +2637,11 @@
         <v>31</v>
       </c>
       <c r="E54" s="41" t="n">
-        <v>1087041</v>
+        <v>1086365</v>
       </c>
       <c r="F54" s="41" t="inlineStr">
         <is>
-          <t>陳族元 連續 31 天加碼 2308 (累計 1,087,041 萬)</t>
+          <t>陳族元 連續 31 天加碼 2308 (累計 1,086,365 萬)</t>
         </is>
       </c>
     </row>
@@ -2831,7 +2835,7 @@
         </is>
       </c>
       <c r="C63" s="34" t="n">
-        <v>1175960</v>
+        <v>1173125</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
@@ -2855,10 +2859,10 @@
         </is>
       </c>
       <c r="I63" s="34" t="n">
-        <v>60746</v>
+        <v>61425</v>
       </c>
       <c r="J63" s="213" t="n">
-        <v>0.380995632335176</v>
+        <v>0.3824956871588917</v>
       </c>
     </row>
     <row r="64">
@@ -3271,7 +3275,7 @@
     <row r="76" ht="22" customHeight="1">
       <c r="B76" s="59" t="inlineStr">
         <is>
-          <t>▍ G. 注意股 (資料日 20261001)</t>
+          <t>▍ G. 注意股 (資料日 20261002)</t>
         </is>
       </c>
     </row>
@@ -3667,7 +3671,7 @@
     <row r="98" ht="22" customHeight="1">
       <c r="B98" s="67" t="inlineStr">
         <is>
-          <t>▍ I. 未來 30 天除權息 (有效 32 檔, 已剔除過期)</t>
+          <t>▍ I. 未來 30 天除權息 (有效 57 檔, 已剔除過期)</t>
         </is>
       </c>
     </row>
@@ -3701,42 +3705,42 @@
     <row r="100">
       <c r="B100" t="inlineStr">
         <is>
-          <t>20261001</t>
+          <t>20261002</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>2323</t>
+          <t>6834</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>中環</t>
+          <t>天二科技</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>息</t>
+          <t>權</t>
         </is>
       </c>
       <c r="F100" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="101">
       <c r="B101" s="41" t="inlineStr">
         <is>
-          <t>20261001</t>
+          <t>20261005</t>
         </is>
       </c>
       <c r="C101" s="41" t="inlineStr">
         <is>
-          <t>9927</t>
+          <t>00406A</t>
         </is>
       </c>
       <c r="D101" s="41" t="inlineStr">
         <is>
-          <t>泰銘</t>
+          <t>主動中信台灣收益</t>
         </is>
       </c>
       <c r="E101" s="41" t="inlineStr">
@@ -3745,32 +3749,32 @@
         </is>
       </c>
       <c r="F101" s="41" t="n">
-        <v>5</v>
+        <v>0.138</v>
       </c>
     </row>
     <row r="102">
       <c r="B102" t="inlineStr">
         <is>
-          <t>20261002</t>
+          <t>20261005</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>6834</t>
+          <t>00939</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>天二科技</t>
+          <t>統一台灣高息動能</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>權</t>
+          <t>息</t>
         </is>
       </c>
       <c r="F102" t="n">
-        <v>0</v>
+        <v>0.125</v>
       </c>
     </row>
     <row r="103">
@@ -3781,12 +3785,12 @@
       </c>
       <c r="C103" s="41" t="inlineStr">
         <is>
-          <t>00406A</t>
+          <t>00984D</t>
         </is>
       </c>
       <c r="D103" s="41" t="inlineStr">
         <is>
-          <t>主動中信台灣收益</t>
+          <t>主動聯博全球非投</t>
         </is>
       </c>
       <c r="E103" s="41" t="inlineStr">
@@ -3794,102 +3798,104 @@
           <t>息</t>
         </is>
       </c>
-      <c r="F103" s="41" t="n"/>
+      <c r="F103" s="41" t="n">
+        <v>0.08500000000000001</v>
+      </c>
     </row>
     <row r="104">
       <c r="B104" t="inlineStr">
         <is>
-          <t>20261005</t>
+          <t>20261006</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>00939</t>
+          <t>2614</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>統一台灣高息動能</t>
+          <t>東森</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>息</t>
-        </is>
+          <t>權息</t>
+        </is>
+      </c>
+      <c r="F104" t="n">
+        <v>0.4</v>
       </c>
     </row>
     <row r="105">
       <c r="B105" s="41" t="inlineStr">
         <is>
-          <t>20261005</t>
+          <t>20261006</t>
         </is>
       </c>
       <c r="C105" s="41" t="inlineStr">
         <is>
-          <t>00984D</t>
+          <t>8021</t>
         </is>
       </c>
       <c r="D105" s="41" t="inlineStr">
         <is>
-          <t>主動聯博全球非投</t>
+          <t>尖點</t>
         </is>
       </c>
       <c r="E105" s="41" t="inlineStr">
         <is>
-          <t>息</t>
-        </is>
-      </c>
-      <c r="F105" s="41" t="n"/>
+          <t>權</t>
+        </is>
+      </c>
+      <c r="F105" s="41" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="106">
       <c r="B106" t="inlineStr">
         <is>
-          <t>20261006</t>
+          <t>20261007</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>2614</t>
+          <t>00940</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>東森</t>
+          <t>元大台灣價值高息</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>權息</t>
-        </is>
-      </c>
-      <c r="F106" t="n">
-        <v>0.4</v>
+          <t>息</t>
+        </is>
       </c>
     </row>
     <row r="107">
       <c r="B107" s="41" t="inlineStr">
         <is>
-          <t>20261006</t>
+          <t>20261007</t>
         </is>
       </c>
       <c r="C107" s="41" t="inlineStr">
         <is>
-          <t>8021</t>
+          <t>00946</t>
         </is>
       </c>
       <c r="D107" s="41" t="inlineStr">
         <is>
-          <t>尖點</t>
+          <t>群益科技高息成長</t>
         </is>
       </c>
       <c r="E107" s="41" t="inlineStr">
         <is>
-          <t>權</t>
-        </is>
-      </c>
-      <c r="F107" s="41" t="n">
-        <v>0</v>
-      </c>
+          <t>息</t>
+        </is>
+      </c>
+      <c r="F107" s="41" t="n"/>
     </row>
     <row r="108">
       <c r="B108" t="inlineStr">
@@ -3899,12 +3905,12 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>00940</t>
+          <t>00953B</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>元大台灣價值高息</t>
+          <t>群益優選非投等債</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -3921,12 +3927,12 @@
       </c>
       <c r="C109" s="41" t="inlineStr">
         <is>
-          <t>00946</t>
+          <t>00985B</t>
         </is>
       </c>
       <c r="D109" s="41" t="inlineStr">
         <is>
-          <t>群益科技高息成長</t>
+          <t>群益ESG投等債0-5</t>
         </is>
       </c>
       <c r="E109" s="41" t="inlineStr">
@@ -3944,18 +3950,21 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>00953B</t>
+          <t>2890</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>群益優選非投等債</t>
+          <t>永豐金</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>息</t>
-        </is>
+          <t>權</t>
+        </is>
+      </c>
+      <c r="F110" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="111">
@@ -3966,12 +3975,12 @@
       </c>
       <c r="C111" s="41" t="inlineStr">
         <is>
-          <t>00985B</t>
+          <t>6108</t>
         </is>
       </c>
       <c r="D111" s="41" t="inlineStr">
         <is>
-          <t>群益ESG投等債0-5</t>
+          <t>競國</t>
         </is>
       </c>
       <c r="E111" s="41" t="inlineStr">
@@ -3979,7 +3988,9 @@
           <t>息</t>
         </is>
       </c>
-      <c r="F111" s="41" t="n"/>
+      <c r="F111" s="41" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="112">
       <c r="B112" t="inlineStr">
@@ -3989,37 +4000,37 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>2890</t>
+          <t>6947</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>永豐金</t>
+          <t>台鎔科技</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>權</t>
+          <t>息</t>
         </is>
       </c>
       <c r="F112" t="n">
-        <v>0</v>
+        <v>0.533326</v>
       </c>
     </row>
     <row r="113">
       <c r="B113" s="41" t="inlineStr">
         <is>
-          <t>20261007</t>
+          <t>20261008</t>
         </is>
       </c>
       <c r="C113" s="41" t="inlineStr">
         <is>
-          <t>6108</t>
+          <t>00400A</t>
         </is>
       </c>
       <c r="D113" s="41" t="inlineStr">
         <is>
-          <t>競國</t>
+          <t>主動國泰動能高息</t>
         </is>
       </c>
       <c r="E113" s="41" t="inlineStr">
@@ -4027,33 +4038,31 @@
           <t>息</t>
         </is>
       </c>
-      <c r="F113" s="41" t="n">
-        <v>1</v>
-      </c>
+      <c r="F113" s="41" t="n"/>
     </row>
     <row r="114">
       <c r="B114" t="inlineStr">
         <is>
-          <t>20261007</t>
+          <t>20261012</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>6947</t>
+          <t>1449</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>台鎔科技</t>
+          <t>佳和</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>息</t>
+          <t>權</t>
         </is>
       </c>
       <c r="F114" t="n">
-        <v>0.533326</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -4327,9 +4336,9 @@
       </c>
     </row>
     <row r="25">
-      <c r="C25" s="73" t="inlineStr">
-        <is>
-          <t>除權息 2 檔 (2323 / 9927)</t>
+      <c r="C25" s="75" t="inlineStr">
+        <is>
+          <t>今日無除權息</t>
         </is>
       </c>
     </row>
@@ -4350,7 +4359,7 @@
     <row r="29" ht="22" customHeight="1">
       <c r="C29" s="77" t="inlineStr">
         <is>
-          <t>-113 億 淨買</t>
+          <t>-111 億 淨買</t>
         </is>
       </c>
     </row>
@@ -14894,29 +14903,29 @@
       </c>
       <c r="D190" s="138" t="inlineStr">
         <is>
-          <t>高力(8996)</t>
+          <t>金居(8358)</t>
         </is>
       </c>
       <c r="E190" s="139" t="n">
-        <v>32</v>
+        <v>68</v>
       </c>
       <c r="F190" s="139" t="n">
-        <v>2</v>
+        <v>60</v>
       </c>
       <c r="G190" s="139" t="n">
-        <v>5027</v>
+        <v>3437</v>
       </c>
       <c r="H190" s="139" t="n">
-        <v>310</v>
+        <v>3030</v>
       </c>
       <c r="I190" s="139" t="n">
-        <v>4717</v>
+        <v>407</v>
       </c>
       <c r="J190" s="140" t="n">
-        <v>1570.94</v>
+        <v>505.4</v>
       </c>
       <c r="K190" s="140" t="n">
-        <v>1552.5</v>
+        <v>504.92</v>
       </c>
       <c r="L190" s="233">
         <f>F190*(K190-J190)</f>
@@ -14929,31 +14938,31 @@
       <c r="C191" s="141" t="n"/>
       <c r="D191" s="138" t="inlineStr">
         <is>
-          <t>友達(2409)</t>
+          <t>合晶(6182)</t>
         </is>
       </c>
       <c r="E191" s="139" t="n">
-        <v>966</v>
+        <v>203</v>
       </c>
       <c r="F191" s="139" t="n">
-        <v>890</v>
+        <v>150</v>
       </c>
       <c r="G191" s="139" t="n">
-        <v>3700</v>
+        <v>2639</v>
       </c>
       <c r="H191" s="139" t="n">
-        <v>3409</v>
+        <v>1944</v>
       </c>
       <c r="I191" s="139" t="n">
-        <v>291</v>
+        <v>695</v>
       </c>
       <c r="J191" s="140" t="n">
-        <v>38.3</v>
+        <v>130</v>
       </c>
       <c r="K191" s="140" t="n">
-        <v>38.3</v>
-      </c>
-      <c r="L191" s="232">
+        <v>129.63</v>
+      </c>
+      <c r="L191" s="233">
         <f>F191*(K191-J191)</f>
         <v/>
       </c>
@@ -14964,29 +14973,29 @@
       <c r="C192" s="141" t="n"/>
       <c r="D192" s="138" t="inlineStr">
         <is>
-          <t>環球晶(6488)</t>
+          <t>禾伸堂(3026)</t>
         </is>
       </c>
       <c r="E192" s="139" t="n">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="F192" s="139" t="n">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="G192" s="139" t="n">
-        <v>3552</v>
+        <v>2391</v>
       </c>
       <c r="H192" s="139" t="n">
-        <v>2943</v>
+        <v>702</v>
       </c>
       <c r="I192" s="139" t="n">
-        <v>609</v>
+        <v>1689</v>
       </c>
       <c r="J192" s="140" t="n">
-        <v>1076.42</v>
+        <v>853.89</v>
       </c>
       <c r="K192" s="140" t="n">
-        <v>1090</v>
+        <v>877</v>
       </c>
       <c r="L192" s="232">
         <f>F192*(K192-J192)</f>
@@ -14999,29 +15008,29 @@
       <c r="C193" s="141" t="n"/>
       <c r="D193" s="138" t="inlineStr">
         <is>
-          <t>亞翔(6139)</t>
+          <t>群創(3481)</t>
         </is>
       </c>
       <c r="E193" s="139" t="n">
-        <v>34</v>
+        <v>446</v>
       </c>
       <c r="F193" s="139" t="n">
-        <v>24</v>
+        <v>331</v>
       </c>
       <c r="G193" s="139" t="n">
-        <v>2590</v>
+        <v>2335</v>
       </c>
       <c r="H193" s="139" t="n">
-        <v>1822</v>
+        <v>1731</v>
       </c>
       <c r="I193" s="139" t="n">
-        <v>768</v>
+        <v>604</v>
       </c>
       <c r="J193" s="140" t="n">
-        <v>761.8200000000001</v>
+        <v>52.35</v>
       </c>
       <c r="K193" s="140" t="n">
-        <v>759.29</v>
+        <v>52.31</v>
       </c>
       <c r="L193" s="233">
         <f>F193*(K193-J193)</f>
@@ -15034,31 +15043,31 @@
       <c r="C194" s="141" t="n"/>
       <c r="D194" s="138" t="inlineStr">
         <is>
-          <t>聯發科(2454)</t>
+          <t>友達(2409)</t>
         </is>
       </c>
       <c r="E194" s="139" t="n">
-        <v>4</v>
+        <v>966</v>
       </c>
       <c r="F194" s="139" t="n">
-        <v>2</v>
+        <v>890</v>
       </c>
       <c r="G194" s="139" t="n">
-        <v>2238</v>
+        <v>2180</v>
       </c>
       <c r="H194" s="139" t="n">
-        <v>1162</v>
+        <v>1458</v>
       </c>
       <c r="I194" s="139" t="n">
-        <v>1076</v>
+        <v>722</v>
       </c>
       <c r="J194" s="140" t="n">
-        <v>5593.75</v>
+        <v>22.57</v>
       </c>
       <c r="K194" s="140" t="n">
-        <v>5810.5</v>
-      </c>
-      <c r="L194" s="232">
+        <v>16.38</v>
+      </c>
+      <c r="L194" s="233">
         <f>F194*(K194-J194)</f>
         <v/>
       </c>
@@ -15079,19 +15088,19 @@
         <v>53</v>
       </c>
       <c r="G195" s="139" t="n">
-        <v>2084</v>
+        <v>2120</v>
       </c>
       <c r="H195" s="139" t="n">
-        <v>1194</v>
+        <v>1195</v>
       </c>
       <c r="I195" s="139" t="n">
-        <v>890</v>
+        <v>925</v>
       </c>
       <c r="J195" s="140" t="n">
-        <v>221.71</v>
+        <v>225.5</v>
       </c>
       <c r="K195" s="140" t="n">
-        <v>225.28</v>
+        <v>225.51</v>
       </c>
       <c r="L195" s="232">
         <f>F195*(K195-J195)</f>
@@ -15104,31 +15113,31 @@
       <c r="C196" s="141" t="n"/>
       <c r="D196" s="138" t="inlineStr">
         <is>
-          <t>旺矽(6223)</t>
+          <t>彩晶(6116)</t>
         </is>
       </c>
       <c r="E196" s="139" t="n">
-        <v>3</v>
+        <v>934</v>
       </c>
       <c r="F196" s="139" t="n">
-        <v>1</v>
+        <v>61</v>
       </c>
       <c r="G196" s="139" t="n">
-        <v>1681</v>
+        <v>1462</v>
       </c>
       <c r="H196" s="139" t="n">
-        <v>58</v>
+        <v>96</v>
       </c>
       <c r="I196" s="139" t="n">
-        <v>1623</v>
+        <v>1366</v>
       </c>
       <c r="J196" s="140" t="n">
-        <v>5604</v>
+        <v>15.65</v>
       </c>
       <c r="K196" s="140" t="n">
-        <v>583</v>
-      </c>
-      <c r="L196" s="233">
+        <v>15.66</v>
+      </c>
+      <c r="L196" s="232">
         <f>F196*(K196-J196)</f>
         <v/>
       </c>
@@ -15139,29 +15148,29 @@
       <c r="C197" s="141" t="n"/>
       <c r="D197" s="138" t="inlineStr">
         <is>
-          <t>台達電(2308)</t>
+          <t>聯發科(2454)</t>
         </is>
       </c>
       <c r="E197" s="139" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="F197" s="139" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G197" s="139" t="n">
-        <v>1674</v>
+        <v>1303</v>
       </c>
       <c r="H197" s="139" t="n">
-        <v>1048</v>
+        <v>1018</v>
       </c>
       <c r="I197" s="139" t="n">
-        <v>626</v>
+        <v>285</v>
       </c>
       <c r="J197" s="140" t="n">
-        <v>1860.56</v>
+        <v>4344.33</v>
       </c>
       <c r="K197" s="140" t="n">
-        <v>2095.4</v>
+        <v>5087.5</v>
       </c>
       <c r="L197" s="232">
         <f>F197*(K197-J197)</f>
@@ -15174,31 +15183,31 @@
       <c r="C198" s="141" t="n"/>
       <c r="D198" s="138" t="inlineStr">
         <is>
-          <t>藥華藥(6446)</t>
+          <t>晶豪科(3006)</t>
         </is>
       </c>
       <c r="E198" s="139" t="n">
-        <v>14</v>
+        <v>46</v>
       </c>
       <c r="F198" s="139" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="G198" s="139" t="n">
-        <v>1671</v>
+        <v>1280</v>
       </c>
       <c r="H198" s="139" t="n">
-        <v>5</v>
+        <v>197</v>
       </c>
       <c r="I198" s="139" t="n">
-        <v>1666</v>
+        <v>1083</v>
       </c>
       <c r="J198" s="140" t="n">
-        <v>1193.64</v>
+        <v>278.24</v>
       </c>
       <c r="K198" s="140" t="n">
-        <v>47</v>
-      </c>
-      <c r="L198" s="233">
+        <v>282</v>
+      </c>
+      <c r="L198" s="232">
         <f>F198*(K198-J198)</f>
         <v/>
       </c>
@@ -15209,31 +15218,31 @@
       <c r="C199" s="141" t="n"/>
       <c r="D199" s="138" t="inlineStr">
         <is>
-          <t>彩晶(6116)</t>
+          <t>鈦昇(8027)</t>
         </is>
       </c>
       <c r="E199" s="139" t="n">
-        <v>934</v>
+        <v>61</v>
       </c>
       <c r="F199" s="139" t="n">
-        <v>61</v>
+        <v>5</v>
       </c>
       <c r="G199" s="139" t="n">
-        <v>1508</v>
+        <v>1278</v>
       </c>
       <c r="H199" s="139" t="n">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="I199" s="139" t="n">
-        <v>1411</v>
+        <v>1173</v>
       </c>
       <c r="J199" s="140" t="n">
-        <v>16.14</v>
+        <v>209.51</v>
       </c>
       <c r="K199" s="140" t="n">
-        <v>15.97</v>
-      </c>
-      <c r="L199" s="233">
+        <v>209.6</v>
+      </c>
+      <c r="L199" s="232">
         <f>F199*(K199-J199)</f>
         <v/>
       </c>
@@ -25714,7 +25723,7 @@
     <row r="485" ht="16.5" customHeight="1">
       <c r="A485" s="205" t="inlineStr">
         <is>
-          <t>ⓘ histock top-buyer 資料 fetched @ 2026-10-01 20:01 | 0/12 success</t>
+          <t>ⓘ histock top-buyer 資料 fetched @ 2026-10-01 20:46 | 0/12 success</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-10-03 03:45
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-10.xlsx
+++ b/data/reports/chip_radar_2026-10.xlsx
@@ -1244,9 +1244,9 @@
     <comment ref="D17" authorId="0" shapeId="0">
       <text>
         <t>⚠️ 假共識警示
-領頭大戶「陳族元」獨佔比 51.4%
-  • 領頭金額 78,193 萬
-  • 合計淨買 152,118 萬
+領頭大戶「陳族元」獨佔比 51.2%
+  • 領頭金額 77,452 萬
+  • 合計淨買 151,377 萬
   • 大戶數 11 位 (名義共識)
 判讀: 名義 11 位大戶共識,
 實質 1 人下注佔 51%,
@@ -1257,12 +1257,12 @@
     <comment ref="D18" authorId="0" shapeId="0">
       <text>
         <t>⚠️ 假共識警示
-領頭大戶「張濬安(航海王)」獨佔比 63.4%
+領頭大戶「張濬安(航海王)」獨佔比 63.6%
   • 領頭金額 37,460 萬
-  • 合計淨買 59,089 萬
+  • 合計淨買 58,893 萬
   • 大戶數 10 位 (名義共識)
 判讀: 名義 10 位大戶共識,
-實質 1 人下注佔 63%,
+實質 1 人下注佔 64%,
 剩餘 9 位為陪襯小單,
 真共識訊號被稀釋.</t>
       </text>
@@ -1770,7 +1770,7 @@
         <v>13</v>
       </c>
       <c r="F16" s="15" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G16" s="16" t="inlineStr">
         <is>
@@ -1786,7 +1786,7 @@
         </is>
       </c>
       <c r="J16" s="18" t="n">
-        <v>42046</v>
+        <v>40472</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
@@ -1800,7 +1800,7 @@
         <v>10</v>
       </c>
       <c r="N16" s="17" t="n">
-        <v>212882</v>
+        <v>211309</v>
       </c>
     </row>
     <row r="17">
@@ -1821,7 +1821,7 @@
         <v>11</v>
       </c>
       <c r="F17" s="15" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G17" s="16" t="inlineStr">
         <is>
@@ -1829,7 +1829,7 @@
         </is>
       </c>
       <c r="H17" s="17" t="n">
-        <v>78193</v>
+        <v>77453</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -1851,7 +1851,7 @@
         <v>8</v>
       </c>
       <c r="N17" s="17" t="n">
-        <v>152118</v>
+        <v>151377</v>
       </c>
     </row>
     <row r="18">
@@ -1902,7 +1902,7 @@
         <v>7</v>
       </c>
       <c r="N18" s="17" t="n">
-        <v>59089</v>
+        <v>58893</v>
       </c>
     </row>
     <row r="19">
@@ -1998,13 +1998,13 @@
         </is>
       </c>
       <c r="L20" s="18" t="n">
-        <v>3016</v>
+        <v>3023</v>
       </c>
       <c r="M20" s="19" t="n">
         <v>9</v>
       </c>
       <c r="N20" s="17" t="n">
-        <v>21372</v>
+        <v>21379</v>
       </c>
     </row>
     <row r="21">
@@ -2025,7 +2025,7 @@
         <v>11</v>
       </c>
       <c r="F21" s="15" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G21" s="16" t="inlineStr">
         <is>
@@ -2055,7 +2055,7 @@
         <v>8</v>
       </c>
       <c r="N21" s="17" t="n">
-        <v>16722</v>
+        <v>17212</v>
       </c>
     </row>
     <row r="22">
@@ -2106,7 +2106,7 @@
         <v>7</v>
       </c>
       <c r="N22" s="17" t="n">
-        <v>15470</v>
+        <v>15440</v>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
@@ -2131,7 +2131,7 @@
         </is>
       </c>
       <c r="G25" s="237" t="n">
-        <v>-50.47234</v>
+        <v>-49.94881</v>
       </c>
     </row>
     <row r="26" ht="28" customHeight="1">
@@ -2149,7 +2149,7 @@
         </is>
       </c>
       <c r="G26" s="239" t="n">
-        <v>0.2269826648936771</v>
+        <v>0.2257934332154343</v>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
@@ -2232,7 +2232,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>38.9%</t>
+          <t>39.1%</t>
         </is>
       </c>
       <c r="F32" t="n">
@@ -2260,11 +2260,11 @@
         </is>
       </c>
       <c r="D33" s="34" t="n">
-        <v>942376</v>
+        <v>911886</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>16.2%</t>
+          <t>15.8%</t>
         </is>
       </c>
       <c r="F33" t="n">
@@ -2276,7 +2276,7 @@
         </is>
       </c>
       <c r="H33" s="34" t="n">
-        <v>260358</v>
+        <v>257653</v>
       </c>
       <c r="I33" s="212" t="n">
         <v>0.0399</v>
@@ -2296,7 +2296,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>10.6%</t>
         </is>
       </c>
       <c r="F34" t="n">
@@ -2308,7 +2308,7 @@
         </is>
       </c>
       <c r="H34" s="34" t="n">
-        <v>212882</v>
+        <v>211309</v>
       </c>
       <c r="I34" s="230" t="n">
         <v>-0.004</v>
@@ -2328,7 +2328,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>9.1%</t>
+          <t>9.2%</t>
         </is>
       </c>
       <c r="F35" t="n">
@@ -2360,7 +2360,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>8.8%</t>
+          <t>8.9%</t>
         </is>
       </c>
       <c r="F36" t="n">
@@ -2765,11 +2765,11 @@
         <v>32</v>
       </c>
       <c r="E56" s="41" t="n">
-        <v>1087288</v>
+        <v>1087224</v>
       </c>
       <c r="F56" s="41" t="inlineStr">
         <is>
-          <t>陳族元 連續 32 天加碼 2308 (累計 1,087,288 萬)</t>
+          <t>陳族元 連續 32 天加碼 2308 (累計 1,087,224 萬)</t>
         </is>
       </c>
     </row>
@@ -2963,7 +2963,7 @@
         </is>
       </c>
       <c r="C65" s="34" t="n">
-        <v>883884</v>
+        <v>854877</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
@@ -2971,7 +2971,7 @@
         </is>
       </c>
       <c r="E65" s="34" t="n">
-        <v>89806</v>
+        <v>86510</v>
       </c>
       <c r="F65" t="inlineStr">
         <is>
@@ -2979,18 +2979,18 @@
         </is>
       </c>
       <c r="G65" s="34" t="n">
-        <v>89623</v>
+        <v>80589</v>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>南電(8046)</t>
+          <t>南亞科(2408)</t>
         </is>
       </c>
       <c r="I65" s="34" t="n">
-        <v>56890</v>
+        <v>54572</v>
       </c>
       <c r="J65" s="213" t="n">
-        <v>0.2673644050471312</v>
+        <v>0.259301981454642</v>
       </c>
     </row>
     <row r="66">
@@ -15075,31 +15075,31 @@
       </c>
       <c r="D190" s="138" t="inlineStr">
         <is>
-          <t>國巨*(2327)</t>
+          <t>友達(2409)</t>
         </is>
       </c>
       <c r="E190" s="139" t="n">
-        <v>144</v>
+        <v>1018</v>
       </c>
       <c r="F190" s="139" t="n">
-        <v>101</v>
+        <v>448</v>
       </c>
       <c r="G190" s="139" t="n">
-        <v>9034</v>
+        <v>4072</v>
       </c>
       <c r="H190" s="139" t="n">
-        <v>6329</v>
+        <v>1793</v>
       </c>
       <c r="I190" s="139" t="n">
-        <v>2705</v>
+        <v>2279</v>
       </c>
       <c r="J190" s="140" t="n">
-        <v>627.36</v>
+        <v>40</v>
       </c>
       <c r="K190" s="140" t="n">
-        <v>626.61</v>
-      </c>
-      <c r="L190" s="233">
+        <v>40.02</v>
+      </c>
+      <c r="L190" s="232">
         <f>F190*(K190-J190)</f>
         <v/>
       </c>
@@ -15110,29 +15110,29 @@
       <c r="C191" s="141" t="n"/>
       <c r="D191" s="138" t="inlineStr">
         <is>
-          <t>南電(8046)</t>
+          <t>台光電(2383)</t>
         </is>
       </c>
       <c r="E191" s="139" t="n">
-        <v>32</v>
+        <v>4</v>
       </c>
       <c r="F191" s="139" t="n">
-        <v>27</v>
+        <v>3</v>
       </c>
       <c r="G191" s="139" t="n">
-        <v>4611</v>
+        <v>2162</v>
       </c>
       <c r="H191" s="139" t="n">
-        <v>3991</v>
+        <v>1687</v>
       </c>
       <c r="I191" s="139" t="n">
-        <v>620</v>
+        <v>475</v>
       </c>
       <c r="J191" s="140" t="n">
-        <v>1440.91</v>
+        <v>5404.5</v>
       </c>
       <c r="K191" s="140" t="n">
-        <v>1478.15</v>
+        <v>5624.67</v>
       </c>
       <c r="L191" s="232">
         <f>F191*(K191-J191)</f>
@@ -15145,31 +15145,31 @@
       <c r="C192" s="141" t="n"/>
       <c r="D192" s="138" t="inlineStr">
         <is>
-          <t>友達(2409)</t>
+          <t>統新(6426)</t>
         </is>
       </c>
       <c r="E192" s="139" t="n">
-        <v>1018</v>
+        <v>47</v>
       </c>
       <c r="F192" s="139" t="n">
-        <v>448</v>
+        <v>3</v>
       </c>
       <c r="G192" s="139" t="n">
-        <v>4118</v>
+        <v>1735</v>
       </c>
       <c r="H192" s="139" t="n">
-        <v>1812</v>
+        <v>106</v>
       </c>
       <c r="I192" s="139" t="n">
-        <v>2306</v>
+        <v>1629</v>
       </c>
       <c r="J192" s="140" t="n">
-        <v>40.45</v>
+        <v>369.13</v>
       </c>
       <c r="K192" s="140" t="n">
-        <v>40.45</v>
-      </c>
-      <c r="L192" s="232">
+        <v>353.33</v>
+      </c>
+      <c r="L192" s="233">
         <f>F192*(K192-J192)</f>
         <v/>
       </c>
@@ -15180,31 +15180,31 @@
       <c r="C193" s="141" t="n"/>
       <c r="D193" s="138" t="inlineStr">
         <is>
-          <t>聯發科(2454)</t>
+          <t>高力(8996)</t>
         </is>
       </c>
       <c r="E193" s="139" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="F193" s="139" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="G193" s="139" t="n">
-        <v>3296</v>
+        <v>1696</v>
       </c>
       <c r="H193" s="139" t="n">
-        <v>2555</v>
+        <v>1205</v>
       </c>
       <c r="I193" s="139" t="n">
-        <v>741</v>
+        <v>491</v>
       </c>
       <c r="J193" s="140" t="n">
-        <v>4708.43</v>
+        <v>1541.36</v>
       </c>
       <c r="K193" s="140" t="n">
-        <v>5110.6</v>
-      </c>
-      <c r="L193" s="232">
+        <v>1506.25</v>
+      </c>
+      <c r="L193" s="233">
         <f>F193*(K193-J193)</f>
         <v/>
       </c>
@@ -15215,29 +15215,29 @@
       <c r="C194" s="141" t="n"/>
       <c r="D194" s="138" t="inlineStr">
         <is>
-          <t>汎銓(6830)</t>
+          <t>矽統(2363)</t>
         </is>
       </c>
       <c r="E194" s="139" t="n">
-        <v>60</v>
+        <v>242</v>
       </c>
       <c r="F194" s="139" t="n">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="G194" s="139" t="n">
-        <v>3272</v>
+        <v>1503</v>
       </c>
       <c r="H194" s="139" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="I194" s="139" t="n">
-        <v>3272</v>
+        <v>1203</v>
       </c>
       <c r="J194" s="140" t="n">
-        <v>545.28</v>
+        <v>62.12</v>
       </c>
       <c r="K194" s="140" t="n">
-        <v>0</v>
+        <v>62.52</v>
       </c>
       <c r="L194" s="232">
         <f>F194*(K194-J194)</f>
@@ -15250,31 +15250,31 @@
       <c r="C195" s="141" t="n"/>
       <c r="D195" s="138" t="inlineStr">
         <is>
-          <t>禾伸堂(3026)</t>
+          <t>嘉澤(3533)</t>
         </is>
       </c>
       <c r="E195" s="139" t="n">
-        <v>36</v>
+        <v>8</v>
       </c>
       <c r="F195" s="139" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="G195" s="139" t="n">
-        <v>3002</v>
+        <v>1472</v>
       </c>
       <c r="H195" s="139" t="n">
-        <v>2307</v>
+        <v>220</v>
       </c>
       <c r="I195" s="139" t="n">
-        <v>695</v>
+        <v>1252</v>
       </c>
       <c r="J195" s="140" t="n">
-        <v>833.83</v>
+        <v>1839.88</v>
       </c>
       <c r="K195" s="140" t="n">
-        <v>823.9299999999999</v>
-      </c>
-      <c r="L195" s="233">
+        <v>2205</v>
+      </c>
+      <c r="L195" s="232">
         <f>F195*(K195-J195)</f>
         <v/>
       </c>
@@ -15285,29 +15285,29 @@
       <c r="C196" s="141" t="n"/>
       <c r="D196" s="138" t="inlineStr">
         <is>
-          <t>台虹(8039)</t>
+          <t>奇鋐(3017)</t>
         </is>
       </c>
       <c r="E196" s="139" t="n">
-        <v>101</v>
+        <v>4</v>
       </c>
       <c r="F196" s="139" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="G196" s="139" t="n">
-        <v>2998</v>
+        <v>1404</v>
       </c>
       <c r="H196" s="139" t="n">
-        <v>260</v>
+        <v>1031</v>
       </c>
       <c r="I196" s="139" t="n">
-        <v>2738</v>
+        <v>373</v>
       </c>
       <c r="J196" s="140" t="n">
-        <v>296.85</v>
+        <v>3509.75</v>
       </c>
       <c r="K196" s="140" t="n">
-        <v>288.67</v>
+        <v>3436.67</v>
       </c>
       <c r="L196" s="233">
         <f>F196*(K196-J196)</f>
@@ -15320,29 +15320,29 @@
       <c r="C197" s="141" t="n"/>
       <c r="D197" s="138" t="inlineStr">
         <is>
-          <t>騰輝電子-KY(6672)</t>
+          <t>晶豪科(3006)</t>
         </is>
       </c>
       <c r="E197" s="139" t="n">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="F197" s="139" t="n">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="G197" s="139" t="n">
-        <v>2068</v>
+        <v>1028</v>
       </c>
       <c r="H197" s="139" t="n">
-        <v>1324</v>
+        <v>612</v>
       </c>
       <c r="I197" s="139" t="n">
-        <v>744</v>
+        <v>416</v>
       </c>
       <c r="J197" s="140" t="n">
-        <v>440.02</v>
+        <v>285.56</v>
       </c>
       <c r="K197" s="140" t="n">
-        <v>441.4</v>
+        <v>291.62</v>
       </c>
       <c r="L197" s="232">
         <f>F197*(K197-J197)</f>
@@ -15355,29 +15355,29 @@
       <c r="C198" s="141" t="n"/>
       <c r="D198" s="138" t="inlineStr">
         <is>
-          <t>統新(6426)</t>
+          <t>群聯(8299)</t>
         </is>
       </c>
       <c r="E198" s="139" t="n">
-        <v>47</v>
+        <v>4</v>
       </c>
       <c r="F198" s="139" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G198" s="139" t="n">
-        <v>1699</v>
+        <v>934</v>
       </c>
       <c r="H198" s="139" t="n">
-        <v>108</v>
+        <v>424</v>
       </c>
       <c r="I198" s="139" t="n">
-        <v>1591</v>
+        <v>510</v>
       </c>
       <c r="J198" s="140" t="n">
-        <v>361.49</v>
+        <v>2334.75</v>
       </c>
       <c r="K198" s="140" t="n">
-        <v>361.33</v>
+        <v>2120.5</v>
       </c>
       <c r="L198" s="233">
         <f>F198*(K198-J198)</f>
@@ -15390,31 +15390,31 @@
       <c r="C199" s="141" t="n"/>
       <c r="D199" s="138" t="inlineStr">
         <is>
-          <t>台積電(2330)</t>
+          <t>營邦(3693)</t>
         </is>
       </c>
       <c r="E199" s="139" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="F199" s="139" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G199" s="139" t="n">
-        <v>1640</v>
+        <v>866</v>
       </c>
       <c r="H199" s="139" t="n">
-        <v>68</v>
+        <v>0</v>
       </c>
       <c r="I199" s="139" t="n">
-        <v>1572</v>
+        <v>866</v>
       </c>
       <c r="J199" s="140" t="n">
-        <v>2343.57</v>
+        <v>666</v>
       </c>
       <c r="K199" s="140" t="n">
-        <v>675</v>
-      </c>
-      <c r="L199" s="233">
+        <v>0</v>
+      </c>
+      <c r="L199" s="232">
         <f>F199*(K199-J199)</f>
         <v/>
       </c>
@@ -25979,7 +25979,7 @@
     <row r="485" ht="16.5" customHeight="1">
       <c r="A485" s="205" t="inlineStr">
         <is>
-          <t>ⓘ histock top-buyer 資料 fetched @ 2026-10-02 18:41 | 0/17 success</t>
+          <t>ⓘ histock top-buyer 資料 fetched @ 2026-10-02 19:45 | 0/17 success</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-10-03 04:23
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-10.xlsx
+++ b/data/reports/chip_radar_2026-10.xlsx
@@ -1244,9 +1244,9 @@
     <comment ref="D17" authorId="0" shapeId="0">
       <text>
         <t>⚠️ 假共識警示
-領頭大戶「陳族元」獨佔比 51.2%
-  • 領頭金額 77,452 萬
-  • 合計淨買 151,377 萬
+領頭大戶「陳族元」獨佔比 51.4%
+  • 領頭金額 78,193 萬
+  • 合計淨買 152,118 萬
   • 大戶數 11 位 (名義共識)
 判讀: 名義 11 位大戶共識,
 實質 1 人下注佔 51%,
@@ -1257,12 +1257,12 @@
     <comment ref="D18" authorId="0" shapeId="0">
       <text>
         <t>⚠️ 假共識警示
-領頭大戶「張濬安(航海王)」獨佔比 63.6%
+領頭大戶「張濬安(航海王)」獨佔比 63.4%
   • 領頭金額 37,460 萬
-  • 合計淨買 58,893 萬
+  • 合計淨買 59,089 萬
   • 大戶數 10 位 (名義共識)
 判讀: 名義 10 位大戶共識,
-實質 1 人下注佔 64%,
+實質 1 人下注佔 63%,
 剩餘 9 位為陪襯小單,
 真共識訊號被稀釋.</t>
       </text>
@@ -1770,7 +1770,7 @@
         <v>13</v>
       </c>
       <c r="F16" s="15" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G16" s="16" t="inlineStr">
         <is>
@@ -1786,7 +1786,7 @@
         </is>
       </c>
       <c r="J16" s="18" t="n">
-        <v>40472</v>
+        <v>42046</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
@@ -1800,7 +1800,7 @@
         <v>10</v>
       </c>
       <c r="N16" s="17" t="n">
-        <v>211309</v>
+        <v>212882</v>
       </c>
     </row>
     <row r="17">
@@ -1821,7 +1821,7 @@
         <v>11</v>
       </c>
       <c r="F17" s="15" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G17" s="16" t="inlineStr">
         <is>
@@ -1829,7 +1829,7 @@
         </is>
       </c>
       <c r="H17" s="17" t="n">
-        <v>77453</v>
+        <v>78193</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -1851,7 +1851,7 @@
         <v>8</v>
       </c>
       <c r="N17" s="17" t="n">
-        <v>151377</v>
+        <v>152118</v>
       </c>
     </row>
     <row r="18">
@@ -1902,7 +1902,7 @@
         <v>7</v>
       </c>
       <c r="N18" s="17" t="n">
-        <v>58893</v>
+        <v>59089</v>
       </c>
     </row>
     <row r="19">
@@ -1998,13 +1998,13 @@
         </is>
       </c>
       <c r="L20" s="18" t="n">
-        <v>3023</v>
+        <v>3016</v>
       </c>
       <c r="M20" s="19" t="n">
         <v>9</v>
       </c>
       <c r="N20" s="17" t="n">
-        <v>21379</v>
+        <v>21372</v>
       </c>
     </row>
     <row r="21">
@@ -2025,7 +2025,7 @@
         <v>11</v>
       </c>
       <c r="F21" s="15" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G21" s="16" t="inlineStr">
         <is>
@@ -2055,7 +2055,7 @@
         <v>8</v>
       </c>
       <c r="N21" s="17" t="n">
-        <v>17212</v>
+        <v>16722</v>
       </c>
     </row>
     <row r="22">
@@ -2106,7 +2106,7 @@
         <v>7</v>
       </c>
       <c r="N22" s="17" t="n">
-        <v>15440</v>
+        <v>15470</v>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
@@ -2131,7 +2131,7 @@
         </is>
       </c>
       <c r="G25" s="237" t="n">
-        <v>-49.94881</v>
+        <v>-50.47234</v>
       </c>
     </row>
     <row r="26" ht="28" customHeight="1">
@@ -2149,7 +2149,7 @@
         </is>
       </c>
       <c r="G26" s="239" t="n">
-        <v>0.2257934332154343</v>
+        <v>0.2267130505520895</v>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
@@ -2232,7 +2232,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>39.1%</t>
+          <t>38.9%</t>
         </is>
       </c>
       <c r="F32" t="n">
@@ -2260,11 +2260,11 @@
         </is>
       </c>
       <c r="D33" s="34" t="n">
-        <v>911886</v>
+        <v>942376</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>15.8%</t>
+          <t>16.2%</t>
         </is>
       </c>
       <c r="F33" t="n">
@@ -2276,7 +2276,7 @@
         </is>
       </c>
       <c r="H33" s="34" t="n">
-        <v>257653</v>
+        <v>260358</v>
       </c>
       <c r="I33" s="212" t="n">
         <v>0.0399</v>
@@ -2296,7 +2296,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>10.6%</t>
+          <t>10.5%</t>
         </is>
       </c>
       <c r="F34" t="n">
@@ -2308,7 +2308,7 @@
         </is>
       </c>
       <c r="H34" s="34" t="n">
-        <v>211309</v>
+        <v>212882</v>
       </c>
       <c r="I34" s="230" t="n">
         <v>-0.004</v>
@@ -2328,7 +2328,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>9.1%</t>
         </is>
       </c>
       <c r="F35" t="n">
@@ -2360,7 +2360,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>8.9%</t>
+          <t>8.8%</t>
         </is>
       </c>
       <c r="F36" t="n">
@@ -2765,11 +2765,11 @@
         <v>32</v>
       </c>
       <c r="E56" s="41" t="n">
-        <v>1087224</v>
+        <v>1087288</v>
       </c>
       <c r="F56" s="41" t="inlineStr">
         <is>
-          <t>陳族元 連續 32 天加碼 2308 (累計 1,087,224 萬)</t>
+          <t>陳族元 連續 32 天加碼 2308 (累計 1,087,288 萬)</t>
         </is>
       </c>
     </row>
@@ -2963,7 +2963,7 @@
         </is>
       </c>
       <c r="C65" s="34" t="n">
-        <v>854877</v>
+        <v>883884</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
@@ -2971,7 +2971,7 @@
         </is>
       </c>
       <c r="E65" s="34" t="n">
-        <v>86510</v>
+        <v>89806</v>
       </c>
       <c r="F65" t="inlineStr">
         <is>
@@ -2979,18 +2979,18 @@
         </is>
       </c>
       <c r="G65" s="34" t="n">
-        <v>80589</v>
+        <v>89623</v>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>南亞科(2408)</t>
+          <t>南電(8046)</t>
         </is>
       </c>
       <c r="I65" s="34" t="n">
-        <v>54572</v>
+        <v>56890</v>
       </c>
       <c r="J65" s="213" t="n">
-        <v>0.259301981454642</v>
+        <v>0.2673644050471312</v>
       </c>
     </row>
     <row r="66">
@@ -15075,31 +15075,31 @@
       </c>
       <c r="D190" s="138" t="inlineStr">
         <is>
-          <t>友達(2409)</t>
+          <t>國巨*(2327)</t>
         </is>
       </c>
       <c r="E190" s="139" t="n">
-        <v>1018</v>
+        <v>144</v>
       </c>
       <c r="F190" s="139" t="n">
-        <v>448</v>
+        <v>101</v>
       </c>
       <c r="G190" s="139" t="n">
-        <v>4072</v>
+        <v>9034</v>
       </c>
       <c r="H190" s="139" t="n">
-        <v>1793</v>
+        <v>6329</v>
       </c>
       <c r="I190" s="139" t="n">
-        <v>2279</v>
+        <v>2705</v>
       </c>
       <c r="J190" s="140" t="n">
-        <v>40</v>
+        <v>627.36</v>
       </c>
       <c r="K190" s="140" t="n">
-        <v>40.02</v>
-      </c>
-      <c r="L190" s="232">
+        <v>626.61</v>
+      </c>
+      <c r="L190" s="233">
         <f>F190*(K190-J190)</f>
         <v/>
       </c>
@@ -15110,29 +15110,29 @@
       <c r="C191" s="141" t="n"/>
       <c r="D191" s="138" t="inlineStr">
         <is>
-          <t>台光電(2383)</t>
+          <t>南電(8046)</t>
         </is>
       </c>
       <c r="E191" s="139" t="n">
-        <v>4</v>
+        <v>32</v>
       </c>
       <c r="F191" s="139" t="n">
-        <v>3</v>
+        <v>27</v>
       </c>
       <c r="G191" s="139" t="n">
-        <v>2162</v>
+        <v>4611</v>
       </c>
       <c r="H191" s="139" t="n">
-        <v>1687</v>
+        <v>3991</v>
       </c>
       <c r="I191" s="139" t="n">
-        <v>475</v>
+        <v>620</v>
       </c>
       <c r="J191" s="140" t="n">
-        <v>5404.5</v>
+        <v>1440.91</v>
       </c>
       <c r="K191" s="140" t="n">
-        <v>5624.67</v>
+        <v>1478.15</v>
       </c>
       <c r="L191" s="232">
         <f>F191*(K191-J191)</f>
@@ -15145,31 +15145,31 @@
       <c r="C192" s="141" t="n"/>
       <c r="D192" s="138" t="inlineStr">
         <is>
-          <t>統新(6426)</t>
+          <t>友達(2409)</t>
         </is>
       </c>
       <c r="E192" s="139" t="n">
-        <v>47</v>
+        <v>1018</v>
       </c>
       <c r="F192" s="139" t="n">
-        <v>3</v>
+        <v>448</v>
       </c>
       <c r="G192" s="139" t="n">
-        <v>1735</v>
+        <v>4118</v>
       </c>
       <c r="H192" s="139" t="n">
-        <v>106</v>
+        <v>1812</v>
       </c>
       <c r="I192" s="139" t="n">
-        <v>1629</v>
+        <v>2306</v>
       </c>
       <c r="J192" s="140" t="n">
-        <v>369.13</v>
+        <v>40.45</v>
       </c>
       <c r="K192" s="140" t="n">
-        <v>353.33</v>
-      </c>
-      <c r="L192" s="233">
+        <v>40.45</v>
+      </c>
+      <c r="L192" s="232">
         <f>F192*(K192-J192)</f>
         <v/>
       </c>
@@ -15180,31 +15180,31 @@
       <c r="C193" s="141" t="n"/>
       <c r="D193" s="138" t="inlineStr">
         <is>
-          <t>高力(8996)</t>
+          <t>聯發科(2454)</t>
         </is>
       </c>
       <c r="E193" s="139" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="F193" s="139" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G193" s="139" t="n">
-        <v>1696</v>
+        <v>3296</v>
       </c>
       <c r="H193" s="139" t="n">
-        <v>1205</v>
+        <v>2555</v>
       </c>
       <c r="I193" s="139" t="n">
-        <v>491</v>
+        <v>741</v>
       </c>
       <c r="J193" s="140" t="n">
-        <v>1541.36</v>
+        <v>4708.43</v>
       </c>
       <c r="K193" s="140" t="n">
-        <v>1506.25</v>
-      </c>
-      <c r="L193" s="233">
+        <v>5110.6</v>
+      </c>
+      <c r="L193" s="232">
         <f>F193*(K193-J193)</f>
         <v/>
       </c>
@@ -15215,29 +15215,29 @@
       <c r="C194" s="141" t="n"/>
       <c r="D194" s="138" t="inlineStr">
         <is>
-          <t>矽統(2363)</t>
+          <t>汎銓(6830)</t>
         </is>
       </c>
       <c r="E194" s="139" t="n">
-        <v>242</v>
+        <v>60</v>
       </c>
       <c r="F194" s="139" t="n">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="G194" s="139" t="n">
-        <v>1503</v>
+        <v>3272</v>
       </c>
       <c r="H194" s="139" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="I194" s="139" t="n">
-        <v>1203</v>
+        <v>3272</v>
       </c>
       <c r="J194" s="140" t="n">
-        <v>62.12</v>
+        <v>545.28</v>
       </c>
       <c r="K194" s="140" t="n">
-        <v>62.52</v>
+        <v>0</v>
       </c>
       <c r="L194" s="232">
         <f>F194*(K194-J194)</f>
@@ -15250,31 +15250,31 @@
       <c r="C195" s="141" t="n"/>
       <c r="D195" s="138" t="inlineStr">
         <is>
-          <t>嘉澤(3533)</t>
+          <t>禾伸堂(3026)</t>
         </is>
       </c>
       <c r="E195" s="139" t="n">
-        <v>8</v>
+        <v>36</v>
       </c>
       <c r="F195" s="139" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="G195" s="139" t="n">
-        <v>1472</v>
+        <v>3002</v>
       </c>
       <c r="H195" s="139" t="n">
-        <v>220</v>
+        <v>2307</v>
       </c>
       <c r="I195" s="139" t="n">
-        <v>1252</v>
+        <v>695</v>
       </c>
       <c r="J195" s="140" t="n">
-        <v>1839.88</v>
+        <v>833.83</v>
       </c>
       <c r="K195" s="140" t="n">
-        <v>2205</v>
-      </c>
-      <c r="L195" s="232">
+        <v>823.9299999999999</v>
+      </c>
+      <c r="L195" s="233">
         <f>F195*(K195-J195)</f>
         <v/>
       </c>
@@ -15285,29 +15285,29 @@
       <c r="C196" s="141" t="n"/>
       <c r="D196" s="138" t="inlineStr">
         <is>
-          <t>奇鋐(3017)</t>
+          <t>台虹(8039)</t>
         </is>
       </c>
       <c r="E196" s="139" t="n">
-        <v>4</v>
+        <v>101</v>
       </c>
       <c r="F196" s="139" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G196" s="139" t="n">
-        <v>1404</v>
+        <v>2998</v>
       </c>
       <c r="H196" s="139" t="n">
-        <v>1031</v>
+        <v>260</v>
       </c>
       <c r="I196" s="139" t="n">
-        <v>373</v>
+        <v>2738</v>
       </c>
       <c r="J196" s="140" t="n">
-        <v>3509.75</v>
+        <v>296.85</v>
       </c>
       <c r="K196" s="140" t="n">
-        <v>3436.67</v>
+        <v>288.67</v>
       </c>
       <c r="L196" s="233">
         <f>F196*(K196-J196)</f>
@@ -15320,29 +15320,29 @@
       <c r="C197" s="141" t="n"/>
       <c r="D197" s="138" t="inlineStr">
         <is>
-          <t>晶豪科(3006)</t>
+          <t>騰輝電子-KY(6672)</t>
         </is>
       </c>
       <c r="E197" s="139" t="n">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="F197" s="139" t="n">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="G197" s="139" t="n">
-        <v>1028</v>
+        <v>2068</v>
       </c>
       <c r="H197" s="139" t="n">
-        <v>612</v>
+        <v>1324</v>
       </c>
       <c r="I197" s="139" t="n">
-        <v>416</v>
+        <v>744</v>
       </c>
       <c r="J197" s="140" t="n">
-        <v>285.56</v>
+        <v>440.02</v>
       </c>
       <c r="K197" s="140" t="n">
-        <v>291.62</v>
+        <v>441.4</v>
       </c>
       <c r="L197" s="232">
         <f>F197*(K197-J197)</f>
@@ -15355,29 +15355,29 @@
       <c r="C198" s="141" t="n"/>
       <c r="D198" s="138" t="inlineStr">
         <is>
-          <t>群聯(8299)</t>
+          <t>統新(6426)</t>
         </is>
       </c>
       <c r="E198" s="139" t="n">
-        <v>4</v>
+        <v>47</v>
       </c>
       <c r="F198" s="139" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G198" s="139" t="n">
-        <v>934</v>
+        <v>1699</v>
       </c>
       <c r="H198" s="139" t="n">
-        <v>424</v>
+        <v>108</v>
       </c>
       <c r="I198" s="139" t="n">
-        <v>510</v>
+        <v>1591</v>
       </c>
       <c r="J198" s="140" t="n">
-        <v>2334.75</v>
+        <v>361.49</v>
       </c>
       <c r="K198" s="140" t="n">
-        <v>2120.5</v>
+        <v>361.33</v>
       </c>
       <c r="L198" s="233">
         <f>F198*(K198-J198)</f>
@@ -15390,31 +15390,31 @@
       <c r="C199" s="141" t="n"/>
       <c r="D199" s="138" t="inlineStr">
         <is>
-          <t>營邦(3693)</t>
+          <t>台積電(2330)</t>
         </is>
       </c>
       <c r="E199" s="139" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="F199" s="139" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G199" s="139" t="n">
-        <v>866</v>
+        <v>1640</v>
       </c>
       <c r="H199" s="139" t="n">
-        <v>0</v>
+        <v>68</v>
       </c>
       <c r="I199" s="139" t="n">
-        <v>866</v>
+        <v>1572</v>
       </c>
       <c r="J199" s="140" t="n">
-        <v>666</v>
+        <v>2343.57</v>
       </c>
       <c r="K199" s="140" t="n">
-        <v>0</v>
-      </c>
-      <c r="L199" s="232">
+        <v>675</v>
+      </c>
+      <c r="L199" s="233">
         <f>F199*(K199-J199)</f>
         <v/>
       </c>
@@ -25979,7 +25979,7 @@
     <row r="485" ht="16.5" customHeight="1">
       <c r="A485" s="205" t="inlineStr">
         <is>
-          <t>ⓘ histock top-buyer 資料 fetched @ 2026-10-02 19:45 | 0/17 success</t>
+          <t>ⓘ histock top-buyer 資料 fetched @ 2026-10-02 20:23 | 0/17 success</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-10-06 05:49
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-10.xlsx
+++ b/data/reports/chip_radar_2026-10.xlsx
@@ -23,7 +23,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="22">
+  <numFmts count="23">
     <numFmt numFmtId="164" formatCode="0%&quot; (13/13 ・昨100/5d100)&quot;"/>
     <numFmt numFmtId="165" formatCode="+0&quot; 億 (昨-42/5d-70)&quot;;-0&quot; 億 (昨-42/5d-70)&quot;;0&quot; 億&quot;"/>
     <numFmt numFmtId="166" formatCode="0&quot; 檔 +11億 &quot;&quot;(昨7/5d12)&quot;"/>
@@ -46,6 +46,7 @@
     <numFmt numFmtId="183" formatCode="+0&quot; 億 (昨-50/5d-75)&quot;;-0&quot; 億 (昨-50/5d-75)&quot;;0&quot; 億&quot;"/>
     <numFmt numFmtId="184" formatCode="0&quot; 檔 +79億 &quot;&quot;(昨7/5d9)&quot;"/>
     <numFmt numFmtId="185" formatCode="0.0%&quot; 市-266億 &quot;&quot;(昨23/5d19)&quot;"/>
+    <numFmt numFmtId="186" formatCode="0.0%&quot; 市-264億 &quot;&quot;(昨23/5d19)&quot;"/>
   </numFmts>
   <fonts count="52">
     <font>
@@ -610,7 +611,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="246">
+  <cellXfs count="247">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1177,6 +1178,9 @@
     <xf numFmtId="172" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="186" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2404,7 +2408,7 @@
         </is>
       </c>
       <c r="G30" s="240" t="n">
-        <v>-83.04103000000001</v>
+        <v>-83.05668</v>
       </c>
     </row>
     <row r="31" ht="28" customHeight="1">
@@ -2421,8 +2425,8 @@
           <t>Q4 追蹤佔比</t>
         </is>
       </c>
-      <c r="G31" s="242" t="n">
-        <v>0.1918231303891946</v>
+      <c r="G31" s="246" t="n">
+        <v>0.1919302925258307</v>
       </c>
     </row>
     <row r="32" ht="22" customHeight="1">
@@ -26251,7 +26255,7 @@
     <row r="485" ht="16.5" customHeight="1">
       <c r="A485" s="205" t="inlineStr">
         <is>
-          <t>ⓘ histock top-buyer 資料 fetched @ 2026-10-05 21:22 | 0/17 success</t>
+          <t>ⓘ histock top-buyer 資料 fetched @ 2026-10-05 21:49 | 0/17 success</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-10-06 06:27
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-10.xlsx
+++ b/data/reports/chip_radar_2026-10.xlsx
@@ -23,7 +23,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="23">
+  <numFmts count="25">
     <numFmt numFmtId="164" formatCode="0%&quot; (13/13 ・昨100/5d100)&quot;"/>
     <numFmt numFmtId="165" formatCode="+0&quot; 億 (昨-42/5d-70)&quot;;-0&quot; 億 (昨-42/5d-70)&quot;;0&quot; 億&quot;"/>
     <numFmt numFmtId="166" formatCode="0&quot; 檔 +11億 &quot;&quot;(昨7/5d12)&quot;"/>
@@ -47,6 +47,8 @@
     <numFmt numFmtId="184" formatCode="0&quot; 檔 +79億 &quot;&quot;(昨7/5d9)&quot;"/>
     <numFmt numFmtId="185" formatCode="0.0%&quot; 市-266億 &quot;&quot;(昨23/5d19)&quot;"/>
     <numFmt numFmtId="186" formatCode="0.0%&quot; 市-264億 &quot;&quot;(昨23/5d19)&quot;"/>
+    <numFmt numFmtId="187" formatCode="0&quot; 檔 +87億 &quot;&quot;(昨7/5d9)&quot;"/>
+    <numFmt numFmtId="188" formatCode="0.0%&quot; 市-263億 &quot;&quot;(昨23/5d19)&quot;"/>
   </numFmts>
   <fonts count="52">
     <font>
@@ -611,7 +613,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="247">
+  <cellXfs count="249">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1181,6 +1183,12 @@
     <xf numFmtId="186" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="187" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="188" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1266,9 +1274,9 @@
     <comment ref="D16" authorId="0" shapeId="0">
       <text>
         <t>⚠️ 假共識警示
-領頭大戶「陳族元」獨佔比 74.6%
-  • 領頭金額 177,499 萬
-  • 合計淨買 237,864 萬
+領頭大戶「陳族元」獨佔比 74.7%
+  • 領頭金額 178,056 萬
+  • 合計淨買 238,421 萬
   • 大戶數 10 位 (名義共識)
 判讀: 名義 10 位大戶共識,
 實質 1 人下注佔 75%,
@@ -1279,13 +1287,26 @@
     <comment ref="D17" authorId="0" shapeId="0">
       <text>
         <t>⚠️ 假共識警示
-領頭大戶「陳族元」獨佔比 77.7%
-  • 領頭金額 115,641 萬
-  • 合計淨買 148,829 萬
+領頭大戶「陳族元」獨佔比 77.8%
+  • 領頭金額 116,584 萬
+  • 合計淨買 149,772 萬
   • 大戶數 11 位 (名義共識)
 判讀: 名義 11 位大戶共識,
 實質 1 人下注佔 78%,
 剩餘 10 位為陪襯小單,
+真共識訊號被稀釋.</t>
+      </text>
+    </comment>
+    <comment ref="D22" authorId="0" shapeId="0">
+      <text>
+        <t>⚠️ 假共識警示
+領頭大戶「張濬安(航海王)」獨佔比 66.3%
+  • 領頭金額 25,142 萬
+  • 合計淨買 37,925 萬
+  • 大戶數 10 位 (名義共識)
+判讀: 名義 10 位大戶共識,
+實質 1 人下注佔 66%,
+剩餘 9 位為陪襯小單,
 真共識訊號被稀釋.</t>
       </text>
     </comment>
@@ -1294,8 +1315,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ConsensusTbl_15" displayName="ConsensusTbl_15" ref="B15:N27" headerRowCount="1">
-  <autoFilter ref="B15:N27"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ConsensusTbl_15" displayName="ConsensusTbl_15" ref="B15:N29" headerRowCount="1">
+  <autoFilter ref="B15:N29"/>
   <tableColumns count="13">
     <tableColumn id="2" name="#"/>
     <tableColumn id="3" name="代號"/>
@@ -1604,7 +1625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:N121"/>
+  <dimension ref="B2:N123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1633,14 +1654,14 @@
     <row r="3" ht="24" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>🎯 12 強共識 / Q5 ↑ 偏多 86.3% / E 10 異常 / F 6 長期 / J 0 集中 / H 3 借券壓力</t>
+          <t>🎯 14 強共識 / Q5 ↑ 偏多 86.3% / E 10 異常 / F 6 長期 / J 0 集中 / H 3 借券壓力</t>
         </is>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>💡 🎯 quad 進場 (78.9% alpha): 2303 / 2327 / 8039 +9  |  避開 — 明日恐處置 3 檔: 3625/4304/4971  |  訊號: 強偏多 (Q5 86.3%, hot=19)</t>
+          <t>💡 🎯 quad 進場 (78.9% alpha): 2303 / 2327 / 8039 +11  |  避開 — 明日恐處置 3 檔: 3625/4304/4971  |  訊號: 強偏多 (Q5 86.3%, hot=19)</t>
         </is>
       </c>
     </row>
@@ -1682,14 +1703,14 @@
     <row r="11" ht="18" customHeight="1">
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>🎯 今日 quad 命中 12 檔 (⭐⭐ 12 premium + ⭐ 0 一般): ⭐⭐聯電(2303), ⭐⭐國巨*(2327), ⭐⭐台虹(8039), ⭐⭐南茂(8150), ⭐⭐京元電子(2449) +7 檔  |  Q5 偏多 + 4 位 master 量爆</t>
+          <t>🎯 今日 quad 命中 14 檔 (⭐⭐ 14 premium + ⭐ 0 一般): ⭐⭐聯電(2303), ⭐⭐國巨*(2327), ⭐⭐台虹(8039), ⭐⭐南茂(8150), ⭐⭐京元電子(2449) +9 檔  |  Q5 偏多 + 4 位 master 量爆</t>
         </is>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>📊 今日共識集中產業 (top 3): 半導體業 5 (42%)  |  光電業 4 (33%)  |  電子零組件業 2 (17%)</t>
+          <t>📊 今日共識集中產業 (top 3): 半導體業 6 (43%)  |  光電業 4 (29%)  |  電子零組件業 3 (21%)</t>
         </is>
       </c>
     </row>
@@ -1800,7 +1821,7 @@
         </is>
       </c>
       <c r="H16" s="17" t="n">
-        <v>177499</v>
+        <v>178056</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -1822,7 +1843,7 @@
         <v>7</v>
       </c>
       <c r="N16" s="17" t="n">
-        <v>237864</v>
+        <v>238421</v>
       </c>
     </row>
     <row r="17">
@@ -1843,7 +1864,7 @@
         <v>11</v>
       </c>
       <c r="F17" s="15" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G17" s="16" t="inlineStr">
         <is>
@@ -1851,7 +1872,7 @@
         </is>
       </c>
       <c r="H17" s="17" t="n">
-        <v>115641</v>
+        <v>116584</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -1873,7 +1894,7 @@
         <v>8</v>
       </c>
       <c r="N17" s="17" t="n">
-        <v>148830</v>
+        <v>149773</v>
       </c>
     </row>
     <row r="18">
@@ -1975,7 +1996,7 @@
         <v>9</v>
       </c>
       <c r="N19" s="17" t="n">
-        <v>94562</v>
+        <v>92915</v>
       </c>
     </row>
     <row r="20">
@@ -1984,49 +2005,49 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>8150</t>
+          <t>2409</t>
         </is>
       </c>
       <c r="D20" s="20" t="inlineStr">
         <is>
-          <t>⭐⭐ 南茂</t>
+          <t>📌 ⭐⭐ 友達</t>
         </is>
       </c>
       <c r="E20" s="14" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F20" s="15" t="n">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="G20" s="16" t="inlineStr">
         <is>
+          <t>張濬安</t>
+        </is>
+      </c>
+      <c r="H20" s="17" t="n">
+        <v>9268</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
           <t>陳族元</t>
         </is>
       </c>
-      <c r="H20" s="17" t="n">
-        <v>19397</v>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>竹科主力分點</t>
-        </is>
-      </c>
       <c r="J20" s="18" t="n">
-        <v>14825</v>
+        <v>8810</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>林滄海</t>
+          <t>強森</t>
         </is>
       </c>
       <c r="L20" s="18" t="n">
-        <v>5293</v>
+        <v>7148</v>
       </c>
       <c r="M20" s="19" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="N20" s="17" t="n">
-        <v>47149</v>
+        <v>47097</v>
       </c>
     </row>
     <row r="21">
@@ -2035,49 +2056,49 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2409</t>
+          <t>8150</t>
         </is>
       </c>
       <c r="D21" s="20" t="inlineStr">
         <is>
-          <t>📌 ⭐⭐ 友達</t>
+          <t>⭐⭐ 南茂</t>
         </is>
       </c>
       <c r="E21" s="14" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F21" s="15" t="n">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="G21" s="16" t="inlineStr">
         <is>
-          <t>張濬安</t>
+          <t>陳族元</t>
         </is>
       </c>
       <c r="H21" s="17" t="n">
-        <v>9268</v>
+        <v>17716</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>陳族元</t>
+          <t>竹科主力分點</t>
         </is>
       </c>
       <c r="J21" s="18" t="n">
-        <v>8755</v>
+        <v>14825</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>強森</t>
+          <t>林滄海</t>
         </is>
       </c>
       <c r="L21" s="18" t="n">
-        <v>7148</v>
+        <v>5293</v>
       </c>
       <c r="M21" s="19" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="N21" s="17" t="n">
-        <v>47042</v>
+        <v>45468</v>
       </c>
     </row>
     <row r="22">
@@ -2086,27 +2107,27 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>8039</t>
-        </is>
-      </c>
-      <c r="D22" s="20" t="inlineStr">
-        <is>
-          <t>📌 ⭐⭐ 台虹</t>
+          <t>6147</t>
+        </is>
+      </c>
+      <c r="D22" s="21" t="inlineStr">
+        <is>
+          <t>📌 ⭐⭐⚠️ 頎邦</t>
         </is>
       </c>
       <c r="E22" s="14" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F22" s="15" t="n">
         <v>15</v>
       </c>
       <c r="G22" s="16" t="inlineStr">
         <is>
-          <t>陳族元</t>
+          <t>張濬安</t>
         </is>
       </c>
       <c r="H22" s="17" t="n">
-        <v>5808</v>
+        <v>25142</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -2114,21 +2135,21 @@
         </is>
       </c>
       <c r="J22" s="18" t="n">
-        <v>3023</v>
+        <v>5751</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>大牌分析師</t>
+          <t>竹科主力分點</t>
         </is>
       </c>
       <c r="L22" s="18" t="n">
-        <v>2932</v>
+        <v>2151</v>
       </c>
       <c r="M22" s="19" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="N22" s="17" t="n">
-        <v>24912</v>
+        <v>37925</v>
       </c>
     </row>
     <row r="23">
@@ -2137,49 +2158,49 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>6488</t>
+          <t>2492</t>
         </is>
       </c>
       <c r="D23" s="20" t="inlineStr">
         <is>
-          <t>⭐⭐ 環球晶</t>
+          <t>📌 ⭐⭐ 華新科</t>
         </is>
       </c>
       <c r="E23" s="14" t="n">
         <v>10</v>
       </c>
       <c r="F23" s="15" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G23" s="16" t="inlineStr">
         <is>
-          <t>陳律師</t>
+          <t>蔣承翰</t>
         </is>
       </c>
       <c r="H23" s="17" t="n">
-        <v>6440</v>
+        <v>10431</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>強森</t>
+          <t>張濬安</t>
         </is>
       </c>
       <c r="J23" s="18" t="n">
-        <v>2741</v>
+        <v>8941</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>陳族元</t>
+          <t>林滄海</t>
         </is>
       </c>
       <c r="L23" s="18" t="n">
-        <v>2719</v>
+        <v>6513</v>
       </c>
       <c r="M23" s="19" t="n">
         <v>7</v>
       </c>
       <c r="N23" s="17" t="n">
-        <v>19559</v>
+        <v>37547</v>
       </c>
     </row>
     <row r="24">
@@ -2188,49 +2209,49 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>6239</t>
+          <t>8039</t>
         </is>
       </c>
       <c r="D24" s="20" t="inlineStr">
         <is>
-          <t>⭐⭐ 力成</t>
+          <t>📌 ⭐⭐ 台虹</t>
         </is>
       </c>
       <c r="E24" s="14" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F24" s="15" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G24" s="16" t="inlineStr">
         <is>
-          <t>強森</t>
+          <t>陳族元</t>
         </is>
       </c>
       <c r="H24" s="17" t="n">
-        <v>3219</v>
+        <v>7458</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>竹科主力分點</t>
+          <t>林滄海</t>
         </is>
       </c>
       <c r="J24" s="18" t="n">
-        <v>3034</v>
+        <v>3023</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>陳族元</t>
+          <t>大牌分析師</t>
         </is>
       </c>
       <c r="L24" s="18" t="n">
-        <v>2709</v>
+        <v>2932</v>
       </c>
       <c r="M24" s="19" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="N24" s="17" t="n">
-        <v>16841</v>
+        <v>26563</v>
       </c>
     </row>
     <row r="25">
@@ -2239,27 +2260,27 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>3481</t>
+          <t>6488</t>
         </is>
       </c>
       <c r="D25" s="20" t="inlineStr">
         <is>
-          <t>⭐⭐ 群創</t>
+          <t>⭐⭐ 環球晶</t>
         </is>
       </c>
       <c r="E25" s="14" t="n">
         <v>10</v>
       </c>
       <c r="F25" s="15" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G25" s="16" t="inlineStr">
         <is>
-          <t>張濬安</t>
+          <t>陳律師</t>
         </is>
       </c>
       <c r="H25" s="17" t="n">
-        <v>5153</v>
+        <v>6440</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -2267,7 +2288,7 @@
         </is>
       </c>
       <c r="J25" s="18" t="n">
-        <v>2642</v>
+        <v>2741</v>
       </c>
       <c r="K25" t="inlineStr">
         <is>
@@ -2275,13 +2296,13 @@
         </is>
       </c>
       <c r="L25" s="18" t="n">
-        <v>2322</v>
+        <v>2719</v>
       </c>
       <c r="M25" s="19" t="n">
         <v>7</v>
       </c>
       <c r="N25" s="17" t="n">
-        <v>16098</v>
+        <v>19559</v>
       </c>
     </row>
     <row r="26">
@@ -2290,19 +2311,19 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2449</t>
+          <t>6239</t>
         </is>
       </c>
       <c r="D26" s="20" t="inlineStr">
         <is>
-          <t>📌 ⭐⭐ 京元電子</t>
+          <t>⭐⭐ 力成</t>
         </is>
       </c>
       <c r="E26" s="14" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F26" s="15" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="G26" s="16" t="inlineStr">
         <is>
@@ -2310,29 +2331,29 @@
         </is>
       </c>
       <c r="H26" s="17" t="n">
-        <v>1842</v>
+        <v>3412</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Tradow</t>
+          <t>強森</t>
         </is>
       </c>
       <c r="J26" s="18" t="n">
-        <v>1043</v>
+        <v>3219</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>強森</t>
+          <t>竹科主力分點</t>
         </is>
       </c>
       <c r="L26" s="18" t="n">
-        <v>799</v>
+        <v>3034</v>
       </c>
       <c r="M26" s="19" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N26" s="17" t="n">
-        <v>7761</v>
+        <v>17544</v>
       </c>
     </row>
     <row r="27">
@@ -2341,35 +2362,35 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>6116</t>
+          <t>3481</t>
         </is>
       </c>
       <c r="D27" s="20" t="inlineStr">
         <is>
-          <t>⭐⭐ 彩晶</t>
+          <t>⭐⭐ 群創</t>
         </is>
       </c>
       <c r="E27" s="14" t="n">
         <v>10</v>
       </c>
       <c r="F27" s="15" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="G27" s="16" t="inlineStr">
         <is>
+          <t>張濬安</t>
+        </is>
+      </c>
+      <c r="H27" s="17" t="n">
+        <v>5153</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
           <t>強森</t>
         </is>
       </c>
-      <c r="H27" s="17" t="n">
-        <v>623</v>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>Tradow</t>
-        </is>
-      </c>
       <c r="J27" s="18" t="n">
-        <v>347</v>
+        <v>2642</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>
@@ -2377,369 +2398,417 @@
         </is>
       </c>
       <c r="L27" s="18" t="n">
-        <v>197</v>
+        <v>2322</v>
       </c>
       <c r="M27" s="19" t="n">
         <v>7</v>
       </c>
       <c r="N27" s="17" t="n">
+        <v>16098</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" t="n">
+        <v>13</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>2449</t>
+        </is>
+      </c>
+      <c r="D28" s="20" t="inlineStr">
+        <is>
+          <t>📌 ⭐⭐ 京元電子</t>
+        </is>
+      </c>
+      <c r="E28" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="F28" s="15" t="n">
+        <v>14</v>
+      </c>
+      <c r="G28" s="16" t="inlineStr">
+        <is>
+          <t>陳族元</t>
+        </is>
+      </c>
+      <c r="H28" s="17" t="n">
+        <v>1842</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Tradow</t>
+        </is>
+      </c>
+      <c r="J28" s="18" t="n">
+        <v>1043</v>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>強森</t>
+        </is>
+      </c>
+      <c r="L28" s="18" t="n">
+        <v>799</v>
+      </c>
+      <c r="M28" s="19" t="n">
+        <v>8</v>
+      </c>
+      <c r="N28" s="17" t="n">
+        <v>7761</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" t="n">
+        <v>14</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>6116</t>
+        </is>
+      </c>
+      <c r="D29" s="20" t="inlineStr">
+        <is>
+          <t>⭐⭐ 彩晶</t>
+        </is>
+      </c>
+      <c r="E29" s="14" t="n">
+        <v>10</v>
+      </c>
+      <c r="F29" s="15" t="n">
+        <v>14</v>
+      </c>
+      <c r="G29" s="16" t="inlineStr">
+        <is>
+          <t>強森</t>
+        </is>
+      </c>
+      <c r="H29" s="17" t="n">
+        <v>623</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Tradow</t>
+        </is>
+      </c>
+      <c r="J29" s="18" t="n">
+        <v>347</v>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>陳族元</t>
+        </is>
+      </c>
+      <c r="L29" s="18" t="n">
+        <v>197</v>
+      </c>
+      <c r="M29" s="19" t="n">
+        <v>7</v>
+      </c>
+      <c r="N29" s="17" t="n">
         <v>1644</v>
       </c>
     </row>
-    <row r="29" ht="22" customHeight="1">
-      <c r="B29" s="22" t="inlineStr">
+    <row r="31" ht="22" customHeight="1">
+      <c r="B31" s="22" t="inlineStr">
         <is>
           <t>▍ A. 追蹤池摘要 (10 秒判讀今日 13 位大戶在做什麼)</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="28" customHeight="1">
-      <c r="B30" s="23" t="inlineStr">
+    <row r="32" ht="28" customHeight="1">
+      <c r="B32" s="23" t="inlineStr">
         <is>
           <t>Q1 活躍率</t>
         </is>
       </c>
-      <c r="C30" s="207" t="n">
+      <c r="C32" s="207" t="n">
         <v>1</v>
       </c>
-      <c r="F30" s="23" t="inlineStr">
+      <c r="F32" s="23" t="inlineStr">
         <is>
           <t>Q2 淨買差</t>
         </is>
       </c>
-      <c r="G30" s="240" t="n">
-        <v>-83.05668</v>
-      </c>
-    </row>
-    <row r="31" ht="28" customHeight="1">
-      <c r="B31" s="23" t="inlineStr">
+      <c r="G32" s="240" t="n">
+        <v>-81.56406</v>
+      </c>
+    </row>
+    <row r="33" ht="28" customHeight="1">
+      <c r="B33" s="23" t="inlineStr">
         <is>
           <t>Q3 強共識股</t>
         </is>
       </c>
-      <c r="C31" s="241" t="n">
-        <v>12</v>
-      </c>
-      <c r="F31" s="23" t="inlineStr">
+      <c r="C33" s="247" t="n">
+        <v>14</v>
+      </c>
+      <c r="F33" s="23" t="inlineStr">
         <is>
           <t>Q4 追蹤佔比</t>
         </is>
       </c>
-      <c r="G31" s="246" t="n">
-        <v>0.1919302925258307</v>
-      </c>
-    </row>
-    <row r="32" ht="22" customHeight="1">
-      <c r="B32" s="28" t="n">
+      <c r="G33" s="248" t="n">
+        <v>0.1914720002753366</v>
+      </c>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="B34" s="28" t="n">
         <v>86.3</v>
       </c>
     </row>
-    <row r="33" ht="18" customHeight="1">
-      <c r="B33" s="29" t="inlineStr">
+    <row r="35" ht="18" customHeight="1">
+      <c r="B35" s="29" t="inlineStr">
         <is>
           <t>✅ 過去 30 天 P/C 命中率: 偏多 14/19 (74%) | 偏空 2/2 (100%) | 整體 16/21 (76%)</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="B35" s="30" t="inlineStr">
+    <row r="37">
+      <c r="B37" s="30" t="inlineStr">
         <is>
           <t>▍ B. Top 5 高手(按今日總買金額)</t>
         </is>
       </c>
-      <c r="F35" s="31" t="inlineStr">
+      <c r="F37" s="31" t="inlineStr">
         <is>
           <t>▍ C. Top 5 熱門個股(按今日淨買金額)</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="B36" s="32" t="inlineStr">
+    <row r="38">
+      <c r="B38" s="32" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="C36" s="32" t="inlineStr">
+      <c r="C38" s="32" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D36" s="32" t="inlineStr">
+      <c r="D38" s="32" t="inlineStr">
         <is>
           <t>買進(萬元)</t>
         </is>
       </c>
-      <c r="E36" s="32" t="inlineStr">
+      <c r="E38" s="32" t="inlineStr">
         <is>
           <t>佔比%</t>
         </is>
       </c>
-      <c r="F36" s="32" t="inlineStr">
+      <c r="F38" s="32" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="G36" s="32" t="inlineStr">
+      <c r="G38" s="32" t="inlineStr">
         <is>
           <t>個股</t>
         </is>
       </c>
-      <c r="H36" s="32" t="inlineStr">
+      <c r="H38" s="32" t="inlineStr">
         <is>
           <t>淨買(萬元)</t>
         </is>
       </c>
-      <c r="I36" s="32" t="inlineStr">
+      <c r="I38" s="32" t="inlineStr">
         <is>
           <t>漲跌%</t>
         </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="B37" t="n">
-        <v>1</v>
-      </c>
-      <c r="C37" s="33" t="inlineStr">
-        <is>
-          <t>張濬安(航海王)</t>
-        </is>
-      </c>
-      <c r="D37" s="34" t="n">
-        <v>2315765</v>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>32.2%</t>
-        </is>
-      </c>
-      <c r="F37" t="n">
-        <v>1</v>
-      </c>
-      <c r="G37" s="16" t="inlineStr">
-        <is>
-          <t>台燿(6274)</t>
-        </is>
-      </c>
-      <c r="H37" s="34" t="n">
-        <v>266019</v>
-      </c>
-      <c r="I37" s="212" t="n">
-        <v>0.09880000000000001</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="B38" t="n">
-        <v>2</v>
-      </c>
-      <c r="C38" s="36" t="inlineStr">
-        <is>
-          <t>陳族元</t>
-        </is>
-      </c>
-      <c r="D38" s="34" t="n">
-        <v>1648933</v>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>22.9%</t>
-        </is>
-      </c>
-      <c r="F38" t="n">
-        <v>2</v>
-      </c>
-      <c r="G38" s="16" t="inlineStr">
-        <is>
-          <t>國巨*(2327)</t>
-        </is>
-      </c>
-      <c r="H38" s="34" t="n">
-        <v>237864</v>
-      </c>
-      <c r="I38" s="243" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="39">
       <c r="B39" t="n">
-        <v>3</v>
-      </c>
-      <c r="C39" s="38" t="inlineStr">
-        <is>
-          <t>林滄海</t>
+        <v>1</v>
+      </c>
+      <c r="C39" s="33" t="inlineStr">
+        <is>
+          <t>張濬安(航海王)</t>
         </is>
       </c>
       <c r="D39" s="34" t="n">
-        <v>904800</v>
+        <v>2315765</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>12.6%</t>
+          <t>32.3%</t>
         </is>
       </c>
       <c r="F39" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G39" s="16" t="inlineStr">
         <is>
-          <t>聯發科(2454)</t>
+          <t>台燿(6274)</t>
         </is>
       </c>
       <c r="H39" s="34" t="n">
-        <v>189978</v>
+        <v>266019</v>
       </c>
       <c r="I39" s="212" t="n">
-        <v>0.0434</v>
+        <v>0.09880000000000001</v>
       </c>
     </row>
     <row r="40">
       <c r="B40" t="n">
-        <v>4</v>
-      </c>
-      <c r="C40" s="51" t="inlineStr">
-        <is>
-          <t>蔣承翰</t>
+        <v>2</v>
+      </c>
+      <c r="C40" s="36" t="inlineStr">
+        <is>
+          <t>陳族元</t>
         </is>
       </c>
       <c r="D40" s="34" t="n">
-        <v>677857</v>
+        <v>1627702</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>9.4%</t>
+          <t>22.7%</t>
         </is>
       </c>
       <c r="F40" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G40" s="16" t="inlineStr">
         <is>
-          <t>南亞(1303)</t>
+          <t>國巨*(2327)</t>
         </is>
       </c>
       <c r="H40" s="34" t="n">
-        <v>178734</v>
-      </c>
-      <c r="I40" s="212" t="n">
-        <v>0.1</v>
+        <v>238421</v>
+      </c>
+      <c r="I40" s="243" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="41">
       <c r="B41" t="n">
+        <v>3</v>
+      </c>
+      <c r="C41" s="38" t="inlineStr">
+        <is>
+          <t>林滄海</t>
+        </is>
+      </c>
+      <c r="D41" s="34" t="n">
+        <v>904800</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>12.6%</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>3</v>
+      </c>
+      <c r="G41" s="16" t="inlineStr">
+        <is>
+          <t>聯發科(2454)</t>
+        </is>
+      </c>
+      <c r="H41" s="34" t="n">
+        <v>189978</v>
+      </c>
+      <c r="I41" s="212" t="n">
+        <v>0.0434</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" t="n">
+        <v>4</v>
+      </c>
+      <c r="C42" s="51" t="inlineStr">
+        <is>
+          <t>蔣承翰</t>
+        </is>
+      </c>
+      <c r="D42" s="34" t="n">
+        <v>677857</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>9.5%</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>4</v>
+      </c>
+      <c r="G42" s="16" t="inlineStr">
+        <is>
+          <t>南亞(1303)</t>
+        </is>
+      </c>
+      <c r="H42" s="34" t="n">
+        <v>178734</v>
+      </c>
+      <c r="I42" s="212" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" t="n">
         <v>5</v>
       </c>
-      <c r="C41" s="37" t="inlineStr">
+      <c r="C43" s="37" t="inlineStr">
         <is>
           <t>陳律師</t>
         </is>
       </c>
-      <c r="D41" s="34" t="n">
+      <c r="D43" s="34" t="n">
         <v>432530</v>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="E43" t="inlineStr">
         <is>
           <t>6.0%</t>
         </is>
       </c>
-      <c r="F41" t="n">
+      <c r="F43" t="n">
         <v>5</v>
       </c>
-      <c r="G41" s="16" t="inlineStr">
+      <c r="G43" s="16" t="inlineStr">
         <is>
           <t>聯亞(3081)</t>
         </is>
       </c>
-      <c r="H41" s="34" t="n">
-        <v>148830</v>
-      </c>
-      <c r="I41" s="212" t="n">
+      <c r="H43" s="34" t="n">
+        <v>149773</v>
+      </c>
+      <c r="I43" s="212" t="n">
         <v>0.0256</v>
       </c>
     </row>
-    <row r="44" ht="22" customHeight="1">
-      <c r="B44" s="40" t="inlineStr">
+    <row r="46" ht="22" customHeight="1">
+      <c r="B46" s="40" t="inlineStr">
         <is>
           <t>▍ E. 異常行為警報 (z&gt;2σ 量爆 + 新標的進場)</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="B45" s="12" t="inlineStr">
+    <row r="47">
+      <c r="B47" s="12" t="inlineStr">
         <is>
           <t>類型</t>
         </is>
       </c>
-      <c r="C45" s="12" t="inlineStr">
+      <c r="C47" s="12" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D45" s="12" t="inlineStr">
+      <c r="D47" s="12" t="inlineStr">
         <is>
           <t>嚴重度</t>
         </is>
       </c>
-      <c r="E45" s="12" t="inlineStr">
+      <c r="E47" s="12" t="inlineStr">
         <is>
           <t>說明</t>
         </is>
       </c>
-      <c r="F45" s="12" t="inlineStr">
+      <c r="F47" s="12" t="inlineStr">
         <is>
           <t>金額/檔數</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>🆕 新標的</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>陳律師</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>陳律師 今日買進 10 檔新標的 (過去從沒買過)</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>10 檔</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="B47" s="41" t="inlineStr">
-        <is>
-          <t>🆕 新標的</t>
-        </is>
-      </c>
-      <c r="C47" s="41" t="inlineStr">
-        <is>
-          <t>張濬安(航海王)</t>
-        </is>
-      </c>
-      <c r="D47" s="41" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="E47" s="41" t="inlineStr">
-        <is>
-          <t>張濬安(航海王) 今日買進 9 檔新標的 (過去從沒買過)</t>
-        </is>
-      </c>
-      <c r="F47" s="41" t="inlineStr">
-        <is>
-          <t>9 檔</t>
         </is>
       </c>
     </row>
@@ -2751,7 +2820,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Tradow</t>
+          <t>陳律師</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2761,12 +2830,12 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Tradow 今日買進 7 檔新標的 (過去從沒買過)</t>
+          <t>陳律師 今日買進 10 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>7 檔</t>
+          <t>10 檔</t>
         </is>
       </c>
     </row>
@@ -2778,7 +2847,7 @@
       </c>
       <c r="C49" s="41" t="inlineStr">
         <is>
-          <t>民哥</t>
+          <t>張濬安(航海王)</t>
         </is>
       </c>
       <c r="D49" s="41" t="inlineStr">
@@ -2788,12 +2857,12 @@
       </c>
       <c r="E49" s="41" t="inlineStr">
         <is>
-          <t>民哥 今日買進 7 檔新標的 (過去從沒買過)</t>
+          <t>張濬安(航海王) 今日買進 9 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F49" s="41" t="inlineStr">
         <is>
-          <t>7 檔</t>
+          <t>9 檔</t>
         </is>
       </c>
     </row>
@@ -2815,12 +2884,12 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>陳族元 今日買進 7 檔新標的 (過去從沒買過)</t>
+          <t>陳族元 今日買進 8 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>7 檔</t>
+          <t>8 檔</t>
         </is>
       </c>
     </row>
@@ -2832,7 +2901,7 @@
       </c>
       <c r="C51" s="41" t="inlineStr">
         <is>
-          <t>強森</t>
+          <t>Tradow</t>
         </is>
       </c>
       <c r="D51" s="41" t="inlineStr">
@@ -2842,12 +2911,12 @@
       </c>
       <c r="E51" s="41" t="inlineStr">
         <is>
-          <t>強森 今日買進 6 檔新標的 (過去從沒買過)</t>
+          <t>Tradow 今日買進 7 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F51" s="41" t="inlineStr">
         <is>
-          <t>6 檔</t>
+          <t>7 檔</t>
         </is>
       </c>
     </row>
@@ -2859,7 +2928,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>竹科主力分點</t>
+          <t>民哥</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2869,12 +2938,12 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>竹科主力分點 今日買進 6 檔新標的 (過去從沒買過)</t>
+          <t>民哥 今日買進 7 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>6 檔</t>
+          <t>7 檔</t>
         </is>
       </c>
     </row>
@@ -2886,7 +2955,7 @@
       </c>
       <c r="C53" s="41" t="inlineStr">
         <is>
-          <t>林滄海</t>
+          <t>強森</t>
         </is>
       </c>
       <c r="D53" s="41" t="inlineStr">
@@ -2896,12 +2965,12 @@
       </c>
       <c r="E53" s="41" t="inlineStr">
         <is>
-          <t>林滄海 今日買進 5 檔新標的 (過去從沒買過)</t>
+          <t>強森 今日買進 6 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F53" s="41" t="inlineStr">
         <is>
-          <t>5 檔</t>
+          <t>6 檔</t>
         </is>
       </c>
     </row>
@@ -2913,7 +2982,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>蔣承翰</t>
+          <t>竹科主力分點</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -2923,128 +2992,136 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>蔣承翰 今日買進 5 檔新標的 (過去從沒買過)</t>
+          <t>竹科主力分點 今日買進 6 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>5 檔</t>
+          <t>6 檔</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="B55" s="41" t="inlineStr">
         <is>
+          <t>🆕 新標的</t>
+        </is>
+      </c>
+      <c r="C55" s="41" t="inlineStr">
+        <is>
+          <t>林滄海</t>
+        </is>
+      </c>
+      <c r="D55" s="41" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E55" s="41" t="inlineStr">
+        <is>
+          <t>林滄海 今日買進 5 檔新標的 (過去從沒買過)</t>
+        </is>
+      </c>
+      <c r="F55" s="41" t="inlineStr">
+        <is>
+          <t>5 檔</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>🆕 新標的</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>蔣承翰</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>蔣承翰 今日買進 5 檔新標的 (過去從沒買過)</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>5 檔</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" s="41" t="inlineStr">
+        <is>
           <t>🔴 量爆</t>
         </is>
       </c>
-      <c r="C55" s="41" t="inlineStr">
+      <c r="C57" s="41" t="inlineStr">
         <is>
           <t>Tradow</t>
         </is>
       </c>
-      <c r="D55" s="41" t="inlineStr">
+      <c r="D57" s="41" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="E55" s="41" t="inlineStr">
+      <c r="E57" s="41" t="inlineStr">
         <is>
           <t>Tradow 今日買進 96,795 萬 (平均 53,204 萬, 偏離 3.3σ)</t>
         </is>
       </c>
-      <c r="F55" s="41" t="n">
+      <c r="F57" s="41" t="n">
         <v>96795</v>
       </c>
     </row>
-    <row r="56">
-      <c r="B56" s="42" t="inlineStr">
+    <row r="58">
+      <c r="B58" s="42" t="inlineStr">
         <is>
           <t>… 另 7 筆 anomaly (詳見當日 sheet)</t>
         </is>
       </c>
-      <c r="C56" s="43" t="n"/>
-      <c r="D56" s="43" t="n"/>
-      <c r="E56" s="43" t="n"/>
-      <c r="F56" s="43" t="n"/>
-    </row>
-    <row r="58" ht="22" customHeight="1">
-      <c r="B58" s="44" t="inlineStr">
+      <c r="C58" s="43" t="n"/>
+      <c r="D58" s="43" t="n"/>
+      <c r="E58" s="43" t="n"/>
+      <c r="F58" s="43" t="n"/>
+    </row>
+    <row r="60" ht="22" customHeight="1">
+      <c r="B60" s="44" t="inlineStr">
         <is>
           <t>▍ F. 跨日連續囤貨 Top 30 (按連續天數排序)</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="B59" s="45" t="inlineStr">
+    <row r="61">
+      <c r="B61" s="45" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="C59" s="45" t="inlineStr">
+      <c r="C61" s="45" t="inlineStr">
         <is>
           <t>股票代號</t>
         </is>
       </c>
-      <c r="D59" s="45" t="inlineStr">
+      <c r="D61" s="45" t="inlineStr">
         <is>
           <t>連續天數</t>
         </is>
       </c>
-      <c r="E59" s="45" t="inlineStr">
+      <c r="E61" s="45" t="inlineStr">
         <is>
           <t>累計買金額(萬)</t>
         </is>
       </c>
-      <c r="F59" s="45" t="inlineStr">
+      <c r="F61" s="45" t="inlineStr">
         <is>
           <t>說明</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>🔴 強森</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>6669</t>
-        </is>
-      </c>
-      <c r="D60" s="46" t="n">
-        <v>41</v>
-      </c>
-      <c r="E60" t="n">
-        <v>240346</v>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>強森 連續 41 天加碼 6669 (累計 240,346 萬)</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="B61" s="41" t="inlineStr">
-        <is>
-          <t>🔴 張濬安(航海王)</t>
-        </is>
-      </c>
-      <c r="C61" s="41" t="inlineStr">
-        <is>
-          <t>2303</t>
-        </is>
-      </c>
-      <c r="D61" s="47" t="n">
-        <v>29</v>
-      </c>
-      <c r="E61" s="41" t="n">
-        <v>1453723</v>
-      </c>
-      <c r="F61" s="41" t="inlineStr">
-        <is>
-          <t>張濬安(航海王) 連續 29 天加碼 2303 (累計 1,453,723 萬)</t>
         </is>
       </c>
     </row>
@@ -3056,18 +3133,18 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>2454</t>
+          <t>6669</t>
         </is>
       </c>
       <c r="D62" s="46" t="n">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="E62" t="n">
-        <v>663011</v>
+        <v>240346</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>強森 連續 29 天加碼 2454 (累計 663,011 萬)</t>
+          <t>強森 連續 41 天加碼 6669 (累計 240,346 萬)</t>
         </is>
       </c>
     </row>
@@ -3079,41 +3156,41 @@
       </c>
       <c r="C63" s="41" t="inlineStr">
         <is>
-          <t>2327</t>
+          <t>2303</t>
         </is>
       </c>
       <c r="D63" s="47" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E63" s="41" t="n">
-        <v>1080516</v>
+        <v>1453723</v>
       </c>
       <c r="F63" s="41" t="inlineStr">
         <is>
-          <t>張濬安(航海王) 連續 28 天加碼 2327 (累計 1,080,516 萬)</t>
+          <t>張濬安(航海王) 連續 29 天加碼 2303 (累計 1,453,723 萬)</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="B64" t="inlineStr">
         <is>
-          <t>🔴 迷你哥/松山哥</t>
+          <t>🔴 強森</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>1303</t>
+          <t>2454</t>
         </is>
       </c>
       <c r="D64" s="46" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E64" t="n">
-        <v>1775127</v>
+        <v>663011</v>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>迷你哥/松山哥 連續 27 天加碼 1303 (累計 1,775,127 萬)</t>
+          <t>強森 連續 29 天加碼 2454 (累計 663,011 萬)</t>
         </is>
       </c>
     </row>
@@ -3125,942 +3202,944 @@
       </c>
       <c r="C65" s="41" t="inlineStr">
         <is>
+          <t>2327</t>
+        </is>
+      </c>
+      <c r="D65" s="47" t="n">
+        <v>28</v>
+      </c>
+      <c r="E65" s="41" t="n">
+        <v>1080516</v>
+      </c>
+      <c r="F65" s="41" t="inlineStr">
+        <is>
+          <t>張濬安(航海王) 連續 28 天加碼 2327 (累計 1,080,516 萬)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>🔴 迷你哥/松山哥</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>1303</t>
+        </is>
+      </c>
+      <c r="D66" s="46" t="n">
+        <v>27</v>
+      </c>
+      <c r="E66" t="n">
+        <v>1775127</v>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>迷你哥/松山哥 連續 27 天加碼 1303 (累計 1,775,127 萬)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" s="41" t="inlineStr">
+        <is>
+          <t>🔴 張濬安(航海王)</t>
+        </is>
+      </c>
+      <c r="C67" s="41" t="inlineStr">
+        <is>
           <t>2454</t>
         </is>
       </c>
-      <c r="D65" s="47" t="n">
+      <c r="D67" s="47" t="n">
         <v>26</v>
       </c>
-      <c r="E65" s="41" t="n">
+      <c r="E67" s="41" t="n">
         <v>1314673</v>
       </c>
-      <c r="F65" s="41" t="inlineStr">
+      <c r="F67" s="41" t="inlineStr">
         <is>
           <t>張濬安(航海王) 連續 26 天加碼 2454 (累計 1,314,673 萬)</t>
         </is>
       </c>
     </row>
-    <row r="67" ht="22" customHeight="1">
-      <c r="B67" s="48" t="inlineStr">
+    <row r="69" ht="22" customHeight="1">
+      <c r="B69" s="48" t="inlineStr">
         <is>
           <t>▍ J. Master × Top 3 個股 cross-table (今日)</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="B68" s="49" t="inlineStr">
+    <row r="70">
+      <c r="B70" s="49" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="C68" s="49" t="inlineStr">
+      <c r="C70" s="49" t="inlineStr">
         <is>
           <t>今日總買(萬)</t>
         </is>
       </c>
-      <c r="D68" s="49" t="inlineStr">
+      <c r="D70" s="49" t="inlineStr">
         <is>
           <t>Top1 個股</t>
         </is>
       </c>
-      <c r="E68" s="49" t="inlineStr">
+      <c r="E70" s="49" t="inlineStr">
         <is>
           <t>Top1 金額</t>
         </is>
       </c>
-      <c r="F68" s="49" t="inlineStr">
+      <c r="F70" s="49" t="inlineStr">
         <is>
           <t>Top2 個股</t>
         </is>
       </c>
-      <c r="G68" s="49" t="inlineStr">
+      <c r="G70" s="49" t="inlineStr">
         <is>
           <t>Top2 金額</t>
         </is>
       </c>
-      <c r="H68" s="49" t="inlineStr">
+      <c r="H70" s="49" t="inlineStr">
         <is>
           <t>Top3 個股</t>
         </is>
       </c>
-      <c r="I68" s="49" t="inlineStr">
+      <c r="I70" s="49" t="inlineStr">
         <is>
           <t>Top3 金額</t>
         </is>
       </c>
-      <c r="J68" s="49" t="inlineStr">
+      <c r="J70" s="49" t="inlineStr">
         <is>
           <t>Top3 合計%</t>
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="B69" s="33" t="inlineStr">
+    <row r="71">
+      <c r="B71" s="33" t="inlineStr">
         <is>
           <t>張濬安(航海王)</t>
         </is>
       </c>
-      <c r="C69" s="34" t="n">
+      <c r="C71" s="34" t="n">
         <v>1648549</v>
       </c>
-      <c r="D69" t="inlineStr">
+      <c r="D71" t="inlineStr">
         <is>
           <t>聯發科(2454)</t>
         </is>
       </c>
-      <c r="E69" s="34" t="n">
+      <c r="E71" s="34" t="n">
         <v>123033</v>
       </c>
-      <c r="F69" t="inlineStr">
+      <c r="F71" t="inlineStr">
         <is>
           <t>台積電(2330)</t>
         </is>
       </c>
-      <c r="G69" s="34" t="n">
+      <c r="G71" s="34" t="n">
         <v>115757</v>
       </c>
-      <c r="H69" t="inlineStr">
+      <c r="H71" t="inlineStr">
         <is>
           <t>台燿(6274)</t>
         </is>
       </c>
-      <c r="I69" s="34" t="n">
+      <c r="I71" s="34" t="n">
         <v>109063</v>
       </c>
-      <c r="J69" s="213" t="n">
+      <c r="J71" s="213" t="n">
         <v>0.2110052665104444</v>
       </c>
     </row>
-    <row r="70">
-      <c r="B70" s="36" t="inlineStr">
+    <row r="72">
+      <c r="B72" s="36" t="inlineStr">
         <is>
           <t>陳族元</t>
         </is>
       </c>
-      <c r="C70" s="34" t="n">
-        <v>1522101</v>
-      </c>
-      <c r="D70" t="inlineStr">
+      <c r="C72" s="34" t="n">
+        <v>1500667</v>
+      </c>
+      <c r="D72" t="inlineStr">
         <is>
           <t>國巨*(2327)</t>
         </is>
       </c>
-      <c r="E70" s="34" t="n">
-        <v>207859</v>
-      </c>
-      <c r="F70" t="inlineStr">
+      <c r="E72" s="34" t="n">
+        <v>205089</v>
+      </c>
+      <c r="F72" t="inlineStr">
         <is>
           <t>金居(8358)</t>
         </is>
       </c>
-      <c r="G70" s="34" t="n">
+      <c r="G72" s="34" t="n">
         <v>137195</v>
       </c>
-      <c r="H70" t="inlineStr">
+      <c r="H72" t="inlineStr">
         <is>
           <t>聯亞(3081)</t>
         </is>
       </c>
-      <c r="I70" s="34" t="n">
-        <v>123776</v>
-      </c>
-      <c r="J70" s="213" t="n">
-        <v>0.3080154843823151</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="B71" s="38" t="inlineStr">
+      <c r="I72" s="34" t="n">
+        <v>125083</v>
+      </c>
+      <c r="J72" s="213" t="n">
+        <v>0.3114398507917111</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="B73" s="38" t="inlineStr">
         <is>
           <t>林滄海</t>
         </is>
       </c>
-      <c r="C71" s="34" t="n">
+      <c r="C73" s="34" t="n">
         <v>882314</v>
       </c>
-      <c r="D71" t="inlineStr">
+      <c r="D73" t="inlineStr">
         <is>
           <t>玉晶光(3406)</t>
         </is>
       </c>
-      <c r="E71" s="34" t="n">
+      <c r="E73" s="34" t="n">
         <v>110171</v>
       </c>
-      <c r="F71" t="inlineStr">
+      <c r="F73" t="inlineStr">
         <is>
           <t>南亞(1303)</t>
         </is>
       </c>
-      <c r="G71" s="34" t="n">
+      <c r="G73" s="34" t="n">
         <v>91439</v>
       </c>
-      <c r="H71" t="inlineStr">
+      <c r="H73" t="inlineStr">
         <is>
           <t>聯發科(2454)</t>
         </is>
       </c>
-      <c r="I71" s="34" t="n">
+      <c r="I73" s="34" t="n">
         <v>88321</v>
       </c>
-      <c r="J71" s="213" t="n">
+      <c r="J73" s="213" t="n">
         <v>0.3286028184294006</v>
       </c>
     </row>
-    <row r="72">
-      <c r="B72" s="51" t="inlineStr">
+    <row r="74">
+      <c r="B74" s="51" t="inlineStr">
         <is>
           <t>蔣承翰</t>
         </is>
       </c>
-      <c r="C72" s="34" t="n">
+      <c r="C74" s="34" t="n">
         <v>603067</v>
       </c>
-      <c r="D72" t="inlineStr">
+      <c r="D74" t="inlineStr">
         <is>
           <t>台燿(6274)</t>
         </is>
       </c>
-      <c r="E72" s="34" t="n">
+      <c r="E74" s="34" t="n">
         <v>126897</v>
       </c>
-      <c r="F72" t="inlineStr">
+      <c r="F74" t="inlineStr">
         <is>
           <t>金像電(2368)</t>
         </is>
       </c>
-      <c r="G72" s="34" t="n">
+      <c r="G74" s="34" t="n">
         <v>61719</v>
       </c>
-      <c r="H72" t="inlineStr">
+      <c r="H74" t="inlineStr">
         <is>
           <t>華通(2313)</t>
         </is>
       </c>
-      <c r="I72" s="34" t="n">
+      <c r="I74" s="34" t="n">
         <v>53623</v>
       </c>
-      <c r="J72" s="213" t="n">
+      <c r="J74" s="213" t="n">
         <v>0.4016804769089466</v>
       </c>
     </row>
-    <row r="73">
-      <c r="B73" s="37" t="inlineStr">
+    <row r="75">
+      <c r="B75" s="37" t="inlineStr">
         <is>
           <t>陳律師</t>
         </is>
       </c>
-      <c r="C73" s="34" t="n">
+      <c r="C75" s="34" t="n">
         <v>425258</v>
       </c>
-      <c r="D73" t="inlineStr">
+      <c r="D75" t="inlineStr">
         <is>
           <t>大立光(3008)</t>
         </is>
       </c>
-      <c r="E73" s="34" t="n">
+      <c r="E75" s="34" t="n">
         <v>59928</v>
       </c>
-      <c r="F73" t="inlineStr">
+      <c r="F75" t="inlineStr">
         <is>
           <t>台燿(6274)</t>
         </is>
       </c>
-      <c r="G73" s="34" t="n">
+      <c r="G75" s="34" t="n">
         <v>48238</v>
       </c>
-      <c r="H73" t="inlineStr">
+      <c r="H75" t="inlineStr">
         <is>
           <t>國巨*(2327)</t>
         </is>
       </c>
-      <c r="I73" s="34" t="n">
+      <c r="I75" s="34" t="n">
         <v>36398</v>
       </c>
-      <c r="J73" s="213" t="n">
+      <c r="J75" s="213" t="n">
         <v>0.3399435166416622</v>
       </c>
     </row>
-    <row r="74">
-      <c r="B74" s="39" t="inlineStr">
+    <row r="76">
+      <c r="B76" s="39" t="inlineStr">
         <is>
           <t>強森</t>
         </is>
       </c>
-      <c r="C74" s="34" t="n">
+      <c r="C76" s="34" t="n">
         <v>376456</v>
       </c>
-      <c r="D74" t="inlineStr">
+      <c r="D76" t="inlineStr">
         <is>
           <t>華邦電(2344)</t>
         </is>
       </c>
-      <c r="E74" s="34" t="n">
+      <c r="E76" s="34" t="n">
         <v>36711</v>
       </c>
-      <c r="F74" t="inlineStr">
+      <c r="F76" t="inlineStr">
         <is>
           <t>創意(3443)</t>
         </is>
       </c>
-      <c r="G74" s="34" t="n">
+      <c r="G76" s="34" t="n">
         <v>27809</v>
       </c>
-      <c r="H74" t="inlineStr">
+      <c r="H76" t="inlineStr">
         <is>
           <t>聯電(2303)</t>
         </is>
       </c>
-      <c r="I74" s="34" t="n">
+      <c r="I76" s="34" t="n">
         <v>27251</v>
       </c>
-      <c r="J74" s="213" t="n">
+      <c r="J76" s="213" t="n">
         <v>0.2437752320458338</v>
       </c>
     </row>
-    <row r="75">
-      <c r="B75" s="52" t="inlineStr">
+    <row r="77">
+      <c r="B77" s="52" t="inlineStr">
         <is>
           <t>民哥</t>
         </is>
       </c>
-      <c r="C75" s="34" t="n">
+      <c r="C77" s="34" t="n">
         <v>178824</v>
       </c>
-      <c r="D75" t="inlineStr">
+      <c r="D77" t="inlineStr">
         <is>
           <t>金居(8358)</t>
         </is>
       </c>
-      <c r="E75" s="34" t="n">
+      <c r="E77" s="34" t="n">
         <v>26191</v>
       </c>
-      <c r="F75" t="inlineStr">
+      <c r="F77" t="inlineStr">
         <is>
           <t>南亞(1303)</t>
         </is>
       </c>
-      <c r="G75" s="34" t="n">
+      <c r="G77" s="34" t="n">
         <v>20014</v>
       </c>
-      <c r="H75" t="inlineStr">
+      <c r="H77" t="inlineStr">
         <is>
           <t>台燿(6274)</t>
         </is>
       </c>
-      <c r="I75" s="34" t="n">
+      <c r="I77" s="34" t="n">
         <v>14898</v>
       </c>
-      <c r="J75" s="213" t="n">
+      <c r="J77" s="213" t="n">
         <v>0.3416920081286537</v>
       </c>
     </row>
-    <row r="76">
-      <c r="B76" s="53" t="inlineStr">
+    <row r="78">
+      <c r="B78" s="53" t="inlineStr">
         <is>
           <t>竹科主力分點</t>
         </is>
       </c>
-      <c r="C76" s="34" t="n">
+      <c r="C78" s="34" t="n">
         <v>156942</v>
       </c>
-      <c r="D76" t="inlineStr">
+      <c r="D78" t="inlineStr">
         <is>
           <t>南茂(8150)</t>
         </is>
       </c>
-      <c r="E76" s="34" t="n">
+      <c r="E78" s="34" t="n">
         <v>16490</v>
       </c>
-      <c r="F76" t="inlineStr">
+      <c r="F78" t="inlineStr">
         <is>
           <t>聯電(2303)</t>
         </is>
       </c>
-      <c r="G76" s="34" t="n">
+      <c r="G78" s="34" t="n">
         <v>15454</v>
       </c>
-      <c r="H76" t="inlineStr">
+      <c r="H78" t="inlineStr">
         <is>
           <t>友達(2409)</t>
         </is>
       </c>
-      <c r="I76" s="34" t="n">
+      <c r="I78" s="34" t="n">
         <v>12563</v>
       </c>
-      <c r="J76" s="213" t="n">
+      <c r="J78" s="213" t="n">
         <v>0.2835833829269629</v>
       </c>
     </row>
-    <row r="77">
-      <c r="B77" s="54" t="inlineStr">
+    <row r="79">
+      <c r="B79" s="54" t="inlineStr">
         <is>
           <t>巨人傑</t>
         </is>
       </c>
-      <c r="C77" s="34" t="n">
+      <c r="C79" s="34" t="n">
         <v>136098</v>
       </c>
-      <c r="D77" t="inlineStr">
+      <c r="D79" t="inlineStr">
         <is>
           <t>台積電(2330)</t>
         </is>
       </c>
-      <c r="E77" s="34" t="n">
+      <c r="E79" s="34" t="n">
         <v>20508</v>
       </c>
-      <c r="F77" t="inlineStr">
+      <c r="F79" t="inlineStr">
         <is>
           <t>台光電(2383)</t>
         </is>
       </c>
-      <c r="G77" s="34" t="n">
+      <c r="G79" s="34" t="n">
         <v>11260</v>
       </c>
-      <c r="H77" t="inlineStr">
+      <c r="H79" t="inlineStr">
         <is>
           <t>強茂(2481)</t>
         </is>
       </c>
-      <c r="I77" s="34" t="n">
+      <c r="I79" s="34" t="n">
         <v>7706</v>
       </c>
-      <c r="J77" s="213" t="n">
+      <c r="J79" s="213" t="n">
         <v>0.2900379431352609</v>
       </c>
     </row>
-    <row r="78">
-      <c r="B78" s="56" t="inlineStr">
+    <row r="80">
+      <c r="B80" s="56" t="inlineStr">
         <is>
           <t>Tradow</t>
         </is>
       </c>
-      <c r="C78" s="34" t="n">
+      <c r="C80" s="34" t="n">
         <v>95352</v>
       </c>
-      <c r="D78" t="inlineStr">
+      <c r="D80" t="inlineStr">
         <is>
           <t>健策(3653)</t>
         </is>
       </c>
-      <c r="E78" s="34" t="n">
+      <c r="E80" s="34" t="n">
         <v>8618</v>
       </c>
-      <c r="F78" t="inlineStr">
+      <c r="F80" t="inlineStr">
         <is>
           <t>聯發科(2454)</t>
         </is>
       </c>
-      <c r="G78" s="34" t="n">
+      <c r="G80" s="34" t="n">
         <v>7417</v>
       </c>
-      <c r="H78" t="inlineStr">
+      <c r="H80" t="inlineStr">
         <is>
           <t>欣興(3037)</t>
         </is>
       </c>
-      <c r="I78" s="34" t="n">
+      <c r="I80" s="34" t="n">
         <v>7330</v>
       </c>
-      <c r="J78" s="213" t="n">
+      <c r="J80" s="213" t="n">
         <v>0.2450428360630465</v>
       </c>
     </row>
-    <row r="79">
-      <c r="B79" s="57" t="inlineStr">
+    <row r="81">
+      <c r="B81" s="57" t="inlineStr">
         <is>
           <t>布哥/n_nchang</t>
         </is>
       </c>
-      <c r="C79" s="34" t="n">
+      <c r="C81" s="34" t="n">
         <v>94495</v>
       </c>
-      <c r="D79" t="inlineStr">
+      <c r="D81" t="inlineStr">
         <is>
           <t>臻鼎-KY(4958)</t>
         </is>
       </c>
-      <c r="E79" s="34" t="n">
+      <c r="E81" s="34" t="n">
         <v>11033</v>
       </c>
-      <c r="F79" t="inlineStr">
+      <c r="F81" t="inlineStr">
         <is>
           <t>健策(3653)</t>
         </is>
       </c>
-      <c r="G79" s="34" t="n">
+      <c r="G81" s="34" t="n">
         <v>7869</v>
       </c>
-      <c r="H79" t="inlineStr">
+      <c r="H81" t="inlineStr">
         <is>
           <t>景碩(3189)</t>
         </is>
       </c>
-      <c r="I79" s="34" t="n">
+      <c r="I81" s="34" t="n">
         <v>6430</v>
       </c>
-      <c r="J79" s="213" t="n">
+      <c r="J81" s="213" t="n">
         <v>0.2680691335239599</v>
       </c>
     </row>
-    <row r="80">
-      <c r="B80" s="55" t="inlineStr">
+    <row r="82">
+      <c r="B82" s="55" t="inlineStr">
         <is>
           <t>大牌分析師</t>
         </is>
       </c>
-      <c r="C80" s="34" t="n">
+      <c r="C82" s="34" t="n">
         <v>89228</v>
       </c>
-      <c r="D80" t="inlineStr">
+      <c r="D82" t="inlineStr">
         <is>
           <t>國巨*(2327)</t>
         </is>
       </c>
-      <c r="E80" s="34" t="n">
+      <c r="E82" s="34" t="n">
         <v>10242</v>
       </c>
-      <c r="F80" t="inlineStr">
+      <c r="F82" t="inlineStr">
         <is>
           <t>聯發科(2454)</t>
         </is>
       </c>
-      <c r="G80" s="34" t="n">
+      <c r="G82" s="34" t="n">
         <v>9456</v>
       </c>
-      <c r="H80" t="inlineStr">
+      <c r="H82" t="inlineStr">
         <is>
           <t>聯電(2303)</t>
         </is>
       </c>
-      <c r="I80" s="34" t="n">
+      <c r="I82" s="34" t="n">
         <v>8038</v>
       </c>
-      <c r="J80" s="213" t="n">
+      <c r="J82" s="213" t="n">
         <v>0.3108560336576717</v>
       </c>
     </row>
-    <row r="81">
-      <c r="B81" s="58" t="inlineStr">
+    <row r="83">
+      <c r="B83" s="58" t="inlineStr">
         <is>
           <t>迷你哥/松山哥</t>
         </is>
       </c>
-      <c r="C81" s="34" t="n">
+      <c r="C83" s="34" t="n">
         <v>23977</v>
       </c>
-      <c r="D81" t="inlineStr">
+      <c r="D83" t="inlineStr">
         <is>
           <t>友達(2409)</t>
         </is>
       </c>
-      <c r="E81" s="34" t="n">
+      <c r="E83" s="34" t="n">
         <v>3639</v>
       </c>
-      <c r="F81" t="inlineStr">
+      <c r="F83" t="inlineStr">
         <is>
           <t>聯電(2303)</t>
         </is>
       </c>
-      <c r="G81" s="34" t="n">
+      <c r="G83" s="34" t="n">
         <v>2785</v>
       </c>
-      <c r="H81" t="inlineStr">
+      <c r="H83" t="inlineStr">
         <is>
           <t>矽格(6257)</t>
         </is>
       </c>
-      <c r="I81" s="34" t="n">
+      <c r="I83" s="34" t="n">
         <v>2032</v>
       </c>
-      <c r="J81" s="213" t="n">
+      <c r="J83" s="213" t="n">
         <v>0.3526715519650327</v>
       </c>
     </row>
-    <row r="83" ht="22" customHeight="1">
-      <c r="B83" s="59" t="inlineStr">
+    <row r="85" ht="22" customHeight="1">
+      <c r="B85" s="59" t="inlineStr">
         <is>
           <t>▍ G. 注意股 (資料日 20261006)</t>
         </is>
       </c>
     </row>
-    <row r="84">
-      <c r="B84" s="60" t="inlineStr">
+    <row r="86">
+      <c r="B86" s="60" t="inlineStr">
         <is>
           <t>代號</t>
         </is>
       </c>
-      <c r="C84" s="60" t="inlineStr">
+      <c r="C86" s="60" t="inlineStr">
         <is>
           <t>名稱</t>
         </is>
       </c>
-      <c r="D84" s="60" t="inlineStr">
+      <c r="D86" s="60" t="inlineStr">
         <is>
           <t>累計次數</t>
         </is>
       </c>
-      <c r="E84" s="60" t="inlineStr">
+      <c r="E86" s="60" t="inlineStr">
         <is>
           <t>收盤價</t>
         </is>
       </c>
-      <c r="F84" s="60" t="inlineStr">
+      <c r="F86" s="60" t="inlineStr">
         <is>
           <t>本益比</t>
         </is>
       </c>
     </row>
-    <row r="85">
-      <c r="B85" s="61" t="inlineStr">
+    <row r="87">
+      <c r="B87" s="61" t="inlineStr">
         <is>
           <t>✅ 今日無新增注意股 (市場無異常波動標的)</t>
         </is>
       </c>
     </row>
-    <row r="87" ht="22" customHeight="1">
-      <c r="B87" s="4" t="inlineStr">
+    <row r="89" ht="22" customHeight="1">
+      <c r="B89" s="4" t="inlineStr">
         <is>
           <t>▍ H. 借券賣出 Top 15 (機構級反向力量, 資料日 20261005)</t>
         </is>
       </c>
     </row>
-    <row r="88">
-      <c r="B88" s="12" t="inlineStr">
+    <row r="90">
+      <c r="B90" s="12" t="inlineStr">
         <is>
           <t>代號</t>
         </is>
       </c>
-      <c r="C88" s="12" t="inlineStr">
+      <c r="C90" s="12" t="inlineStr">
         <is>
           <t>名稱</t>
         </is>
       </c>
-      <c r="D88" s="12" t="inlineStr">
+      <c r="D90" s="12" t="inlineStr">
         <is>
           <t>借券張數</t>
         </is>
       </c>
-      <c r="E88" s="12" t="inlineStr">
+      <c r="E90" s="12" t="inlineStr">
         <is>
           <t>融券張數</t>
         </is>
       </c>
-      <c r="F88" s="12" t="inlineStr">
+      <c r="F90" s="12" t="inlineStr">
         <is>
           <t>ratio</t>
         </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>2409</t>
-        </is>
-      </c>
-      <c r="C89" t="inlineStr">
-        <is>
-          <t>友達</t>
-        </is>
-      </c>
-      <c r="D89" s="34" t="n">
-        <v>27608</v>
-      </c>
-      <c r="E89" s="34" t="n">
-        <v>2843</v>
-      </c>
-      <c r="F89" s="214" t="n">
-        <v>9.710000000000001</v>
-      </c>
-    </row>
-    <row r="90">
-      <c r="B90" s="47" t="inlineStr">
-        <is>
-          <t>🔴 00712</t>
-        </is>
-      </c>
-      <c r="C90" s="41" t="inlineStr">
-        <is>
-          <t>復華富時不動產</t>
-        </is>
-      </c>
-      <c r="D90" s="62" t="n">
-        <v>23161</v>
-      </c>
-      <c r="E90" s="62" t="n">
-        <v>21</v>
-      </c>
-      <c r="F90" s="216" t="n">
-        <v>1102.9</v>
       </c>
     </row>
     <row r="91">
       <c r="B91" t="inlineStr">
         <is>
-          <t>2303</t>
+          <t>2409</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>聯電</t>
+          <t>友達</t>
         </is>
       </c>
       <c r="D91" s="34" t="n">
-        <v>21383</v>
+        <v>27608</v>
       </c>
       <c r="E91" s="34" t="n">
-        <v>50</v>
+        <v>2843</v>
       </c>
       <c r="F91" s="214" t="n">
-        <v>427.66</v>
+        <v>9.710000000000001</v>
       </c>
     </row>
     <row r="92">
-      <c r="B92" s="41" t="inlineStr">
-        <is>
-          <t>3481</t>
+      <c r="B92" s="47" t="inlineStr">
+        <is>
+          <t>🔴 00712</t>
         </is>
       </c>
       <c r="C92" s="41" t="inlineStr">
         <is>
-          <t>群創</t>
+          <t>復華富時不動產</t>
         </is>
       </c>
       <c r="D92" s="62" t="n">
-        <v>15115</v>
+        <v>23161</v>
       </c>
       <c r="E92" s="62" t="n">
-        <v>197</v>
-      </c>
-      <c r="F92" s="215" t="n">
-        <v>76.73</v>
+        <v>21</v>
+      </c>
+      <c r="F92" s="216" t="n">
+        <v>1102.9</v>
       </c>
     </row>
     <row r="93">
       <c r="B93" t="inlineStr">
         <is>
-          <t>2324</t>
+          <t>2303</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>仁寶</t>
+          <t>聯電</t>
         </is>
       </c>
       <c r="D93" s="34" t="n">
-        <v>13147</v>
+        <v>21383</v>
       </c>
       <c r="E93" s="34" t="n">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="F93" s="214" t="n">
-        <v>305.74</v>
+        <v>427.66</v>
       </c>
     </row>
     <row r="94">
       <c r="B94" s="41" t="inlineStr">
         <is>
-          <t>2002</t>
+          <t>3481</t>
         </is>
       </c>
       <c r="C94" s="41" t="inlineStr">
         <is>
-          <t>中鋼</t>
+          <t>群創</t>
         </is>
       </c>
       <c r="D94" s="62" t="n">
-        <v>8001</v>
+        <v>15115</v>
       </c>
       <c r="E94" s="62" t="n">
-        <v>12</v>
+        <v>197</v>
       </c>
       <c r="F94" s="215" t="n">
-        <v>666.75</v>
+        <v>76.73</v>
       </c>
     </row>
     <row r="95">
       <c r="B95" t="inlineStr">
         <is>
-          <t>00405A</t>
+          <t>2324</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>主動富邦台灣龍耀</t>
+          <t>仁寶</t>
         </is>
       </c>
       <c r="D95" s="34" t="n">
-        <v>7000</v>
+        <v>13147</v>
       </c>
       <c r="E95" s="34" t="n">
-        <v>492</v>
+        <v>43</v>
       </c>
       <c r="F95" s="214" t="n">
-        <v>14.23</v>
+        <v>305.74</v>
       </c>
     </row>
     <row r="96">
       <c r="B96" s="41" t="inlineStr">
         <is>
-          <t>00406A</t>
+          <t>2002</t>
         </is>
       </c>
       <c r="C96" s="41" t="inlineStr">
         <is>
-          <t>主動中信台灣收益</t>
+          <t>中鋼</t>
         </is>
       </c>
       <c r="D96" s="62" t="n">
-        <v>6500</v>
+        <v>8001</v>
       </c>
       <c r="E96" s="62" t="n">
-        <v>140</v>
+        <v>12</v>
       </c>
       <c r="F96" s="215" t="n">
-        <v>46.43</v>
+        <v>666.75</v>
       </c>
     </row>
     <row r="97">
-      <c r="B97" s="46" t="inlineStr">
-        <is>
-          <t>🔴 2887</t>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>00405A</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>台新新光金</t>
+          <t>主動富邦台灣龍耀</t>
         </is>
       </c>
       <c r="D97" s="34" t="n">
-        <v>5411</v>
+        <v>7000</v>
       </c>
       <c r="E97" s="34" t="n">
-        <v>5</v>
-      </c>
-      <c r="F97" s="217" t="n">
-        <v>1082.2</v>
+        <v>492</v>
+      </c>
+      <c r="F97" s="214" t="n">
+        <v>14.23</v>
       </c>
     </row>
     <row r="98">
       <c r="B98" s="41" t="inlineStr">
         <is>
-          <t>2812</t>
+          <t>00406A</t>
         </is>
       </c>
       <c r="C98" s="41" t="inlineStr">
         <is>
-          <t>台中銀</t>
+          <t>主動中信台灣收益</t>
         </is>
       </c>
       <c r="D98" s="62" t="n">
-        <v>4555</v>
+        <v>6500</v>
       </c>
       <c r="E98" s="62" t="n">
-        <v>7</v>
+        <v>140</v>
       </c>
       <c r="F98" s="215" t="n">
-        <v>650.71</v>
+        <v>46.43</v>
       </c>
     </row>
     <row r="99">
       <c r="B99" s="46" t="inlineStr">
         <is>
-          <t>🔴 2356</t>
+          <t>🔴 2887</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>英業達</t>
+          <t>台新新光金</t>
         </is>
       </c>
       <c r="D99" s="34" t="n">
-        <v>4289</v>
+        <v>5411</v>
       </c>
       <c r="E99" s="34" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F99" s="217" t="n">
-        <v>2144.5</v>
+        <v>1082.2</v>
       </c>
     </row>
     <row r="100">
       <c r="B100" s="41" t="inlineStr">
         <is>
-          <t>1101</t>
+          <t>2812</t>
         </is>
       </c>
       <c r="C100" s="41" t="inlineStr">
         <is>
-          <t>台泥</t>
+          <t>台中銀</t>
         </is>
       </c>
       <c r="D100" s="62" t="n">
-        <v>4276</v>
+        <v>4555</v>
       </c>
       <c r="E100" s="62" t="n">
-        <v>0</v>
-      </c>
-      <c r="F100" s="41" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>7</v>
+      </c>
+      <c r="F100" s="215" t="n">
+        <v>650.71</v>
       </c>
     </row>
     <row r="101">
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>2801</t>
+      <c r="B101" s="46" t="inlineStr">
+        <is>
+          <t>🔴 2356</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>彰銀</t>
+          <t>英業達</t>
         </is>
       </c>
       <c r="D101" s="34" t="n">
-        <v>4222</v>
+        <v>4289</v>
       </c>
       <c r="E101" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F101" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>2</v>
+      </c>
+      <c r="F101" s="217" t="n">
+        <v>2144.5</v>
       </c>
     </row>
     <row r="102">
       <c r="B102" s="41" t="inlineStr">
         <is>
-          <t>2542</t>
+          <t>1101</t>
         </is>
       </c>
       <c r="C102" s="41" t="inlineStr">
         <is>
-          <t>興富發</t>
+          <t>台泥</t>
         </is>
       </c>
       <c r="D102" s="62" t="n">
-        <v>3346</v>
+        <v>4276</v>
       </c>
       <c r="E102" s="62" t="n">
-        <v>4</v>
-      </c>
-      <c r="F102" s="215" t="n">
-        <v>836.5</v>
+        <v>0</v>
+      </c>
+      <c r="F102" s="41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="103">
       <c r="B103" t="inlineStr">
         <is>
-          <t>009802</t>
+          <t>2801</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>富邦旗艦50</t>
+          <t>彰銀</t>
         </is>
       </c>
       <c r="D103" s="34" t="n">
-        <v>2965</v>
+        <v>4222</v>
       </c>
       <c r="E103" s="34" t="n">
         <v>0</v>
@@ -4071,138 +4150,132 @@
         </is>
       </c>
     </row>
-    <row r="105" ht="22" customHeight="1">
-      <c r="B105" s="67" t="inlineStr">
+    <row r="104">
+      <c r="B104" s="41" t="inlineStr">
+        <is>
+          <t>2542</t>
+        </is>
+      </c>
+      <c r="C104" s="41" t="inlineStr">
+        <is>
+          <t>興富發</t>
+        </is>
+      </c>
+      <c r="D104" s="62" t="n">
+        <v>3346</v>
+      </c>
+      <c r="E104" s="62" t="n">
+        <v>4</v>
+      </c>
+      <c r="F104" s="215" t="n">
+        <v>836.5</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>009802</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>富邦旗艦50</t>
+        </is>
+      </c>
+      <c r="D105" s="34" t="n">
+        <v>2965</v>
+      </c>
+      <c r="E105" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="22" customHeight="1">
+      <c r="B107" s="67" t="inlineStr">
         <is>
           <t>▍ I. 未來 30 天除權息 (有效 58 檔, 已剔除過期)</t>
         </is>
       </c>
     </row>
-    <row r="106">
-      <c r="B106" s="60" t="inlineStr">
+    <row r="108">
+      <c r="B108" s="60" t="inlineStr">
         <is>
           <t>除權息日</t>
         </is>
       </c>
-      <c r="C106" s="60" t="inlineStr">
+      <c r="C108" s="60" t="inlineStr">
         <is>
           <t>代號</t>
         </is>
       </c>
-      <c r="D106" s="60" t="inlineStr">
+      <c r="D108" s="60" t="inlineStr">
         <is>
           <t>名稱</t>
         </is>
       </c>
-      <c r="E106" s="60" t="inlineStr">
+      <c r="E108" s="60" t="inlineStr">
         <is>
           <t>類型</t>
         </is>
       </c>
-      <c r="F106" s="60" t="inlineStr">
+      <c r="F108" s="60" t="inlineStr">
         <is>
           <t>現金股利</t>
         </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>20261006</t>
-        </is>
-      </c>
-      <c r="C107" t="inlineStr">
-        <is>
-          <t>2614</t>
-        </is>
-      </c>
-      <c r="D107" t="inlineStr">
-        <is>
-          <t>東森</t>
-        </is>
-      </c>
-      <c r="E107" t="inlineStr">
-        <is>
-          <t>權息</t>
-        </is>
-      </c>
-      <c r="F107" t="n">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="108">
-      <c r="B108" s="41" t="inlineStr">
-        <is>
-          <t>20261006</t>
-        </is>
-      </c>
-      <c r="C108" s="41" t="inlineStr">
-        <is>
-          <t>8021</t>
-        </is>
-      </c>
-      <c r="D108" s="41" t="inlineStr">
-        <is>
-          <t>尖點</t>
-        </is>
-      </c>
-      <c r="E108" s="41" t="inlineStr">
-        <is>
-          <t>權</t>
-        </is>
-      </c>
-      <c r="F108" s="41" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="109">
       <c r="B109" t="inlineStr">
         <is>
-          <t>20261007</t>
+          <t>20261006</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>00940</t>
+          <t>2614</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>元大台灣價值高息</t>
+          <t>東森</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>息</t>
+          <t>權息</t>
         </is>
       </c>
       <c r="F109" t="n">
-        <v>0.055</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="110">
       <c r="B110" s="41" t="inlineStr">
         <is>
-          <t>20261007</t>
+          <t>20261006</t>
         </is>
       </c>
       <c r="C110" s="41" t="inlineStr">
         <is>
-          <t>00946</t>
+          <t>8021</t>
         </is>
       </c>
       <c r="D110" s="41" t="inlineStr">
         <is>
-          <t>群益科技高息成長</t>
+          <t>尖點</t>
         </is>
       </c>
       <c r="E110" s="41" t="inlineStr">
         <is>
-          <t>息</t>
+          <t>權</t>
         </is>
       </c>
       <c r="F110" s="41" t="n">
-        <v>0.058</v>
+        <v>0</v>
       </c>
     </row>
     <row r="111">
@@ -4213,12 +4286,12 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>00953B</t>
+          <t>00940</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>群益優選非投等債</t>
+          <t>元大台灣價值高息</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -4227,7 +4300,7 @@
         </is>
       </c>
       <c r="F111" t="n">
-        <v>0.067</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="112">
@@ -4238,12 +4311,12 @@
       </c>
       <c r="C112" s="41" t="inlineStr">
         <is>
-          <t>00985B</t>
+          <t>00946</t>
         </is>
       </c>
       <c r="D112" s="41" t="inlineStr">
         <is>
-          <t>群益ESG投等債0-5</t>
+          <t>群益科技高息成長</t>
         </is>
       </c>
       <c r="E112" s="41" t="inlineStr">
@@ -4252,7 +4325,7 @@
         </is>
       </c>
       <c r="F112" s="41" t="n">
-        <v>0.053</v>
+        <v>0.058</v>
       </c>
     </row>
     <row r="113">
@@ -4263,21 +4336,21 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>2890</t>
+          <t>00953B</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>永豐金</t>
+          <t>群益優選非投等債</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>權</t>
+          <t>息</t>
         </is>
       </c>
       <c r="F113" t="n">
-        <v>0</v>
+        <v>0.067</v>
       </c>
     </row>
     <row r="114">
@@ -4288,12 +4361,12 @@
       </c>
       <c r="C114" s="41" t="inlineStr">
         <is>
-          <t>6108</t>
+          <t>00985B</t>
         </is>
       </c>
       <c r="D114" s="41" t="inlineStr">
         <is>
-          <t>競國</t>
+          <t>群益ESG投等債0-5</t>
         </is>
       </c>
       <c r="E114" s="41" t="inlineStr">
@@ -4302,7 +4375,7 @@
         </is>
       </c>
       <c r="F114" s="41" t="n">
-        <v>1</v>
+        <v>0.053</v>
       </c>
     </row>
     <row r="115">
@@ -4313,37 +4386,37 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>6947</t>
+          <t>2890</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>台鎔科技</t>
+          <t>永豐金</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>息</t>
+          <t>權</t>
         </is>
       </c>
       <c r="F115" t="n">
-        <v>0.533326</v>
+        <v>0</v>
       </c>
     </row>
     <row r="116">
       <c r="B116" s="41" t="inlineStr">
         <is>
-          <t>20261008</t>
+          <t>20261007</t>
         </is>
       </c>
       <c r="C116" s="41" t="inlineStr">
         <is>
-          <t>00400A</t>
+          <t>6108</t>
         </is>
       </c>
       <c r="D116" s="41" t="inlineStr">
         <is>
-          <t>主動國泰動能高息</t>
+          <t>競國</t>
         </is>
       </c>
       <c r="E116" s="41" t="inlineStr">
@@ -4352,123 +4425,173 @@
         </is>
       </c>
       <c r="F116" s="41" t="n">
-        <v>0.12</v>
+        <v>1</v>
       </c>
     </row>
     <row r="117">
       <c r="B117" t="inlineStr">
         <is>
-          <t>20261012</t>
+          <t>20261007</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>1449</t>
+          <t>6947</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>佳和</t>
+          <t>台鎔科技</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>權</t>
+          <t>息</t>
         </is>
       </c>
       <c r="F117" t="n">
-        <v>0</v>
+        <v>0.533326</v>
       </c>
     </row>
     <row r="118">
       <c r="B118" s="41" t="inlineStr">
         <is>
-          <t>20261013</t>
+          <t>20261008</t>
         </is>
       </c>
       <c r="C118" s="41" t="inlineStr">
         <is>
-          <t>1727</t>
+          <t>00400A</t>
         </is>
       </c>
       <c r="D118" s="41" t="inlineStr">
         <is>
-          <t>中華化</t>
+          <t>主動國泰動能高息</t>
         </is>
       </c>
       <c r="E118" s="41" t="inlineStr">
         <is>
-          <t>權</t>
+          <t>息</t>
         </is>
       </c>
       <c r="F118" s="41" t="n">
-        <v>0</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="119">
       <c r="B119" t="inlineStr">
         <is>
-          <t>20261015</t>
+          <t>20261012</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>00401A</t>
+          <t>1449</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>主動摩根台灣鑫收</t>
+          <t>佳和</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>息</t>
-        </is>
+          <t>權</t>
+        </is>
+      </c>
+      <c r="F119" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="120">
       <c r="B120" s="41" t="inlineStr">
         <is>
-          <t>20261015</t>
+          <t>20261013</t>
         </is>
       </c>
       <c r="C120" s="41" t="inlineStr">
         <is>
-          <t>1463</t>
+          <t>1727</t>
         </is>
       </c>
       <c r="D120" s="41" t="inlineStr">
         <is>
-          <t>強盛新</t>
+          <t>中華化</t>
         </is>
       </c>
       <c r="E120" s="41" t="inlineStr">
         <is>
-          <t>息</t>
+          <t>權</t>
         </is>
       </c>
       <c r="F120" s="41" t="n">
-        <v>0.1273</v>
+        <v>0</v>
       </c>
     </row>
     <row r="121">
       <c r="B121" t="inlineStr">
         <is>
+          <t>20261015</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>00401A</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>主動摩根台灣鑫收</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>息</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="B122" s="41" t="inlineStr">
+        <is>
+          <t>20261015</t>
+        </is>
+      </c>
+      <c r="C122" s="41" t="inlineStr">
+        <is>
+          <t>1463</t>
+        </is>
+      </c>
+      <c r="D122" s="41" t="inlineStr">
+        <is>
+          <t>強盛新</t>
+        </is>
+      </c>
+      <c r="E122" s="41" t="inlineStr">
+        <is>
+          <t>息</t>
+        </is>
+      </c>
+      <c r="F122" s="41" t="n">
+        <v>0.1273</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="B123" t="inlineStr">
+        <is>
           <t>20261016</t>
         </is>
       </c>
-      <c r="C121" t="inlineStr">
+      <c r="C123" t="inlineStr">
         <is>
           <t>00851</t>
         </is>
       </c>
-      <c r="D121" t="inlineStr">
+      <c r="D123" t="inlineStr">
         <is>
           <t>台新全球AI</t>
         </is>
       </c>
-      <c r="E121" t="inlineStr">
+      <c r="E123" t="inlineStr">
         <is>
           <t>息</t>
         </is>
@@ -4476,37 +4599,37 @@
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="B67:J67"/>
     <mergeCell ref="B9:N9"/>
-    <mergeCell ref="B33:N33"/>
-    <mergeCell ref="G30:I30"/>
-    <mergeCell ref="B56:F56"/>
-    <mergeCell ref="B44:J44"/>
-    <mergeCell ref="B29:J29"/>
-    <mergeCell ref="B87:J87"/>
-    <mergeCell ref="B35:E35"/>
-    <mergeCell ref="B32:N32"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="B107:J107"/>
+    <mergeCell ref="B60:J60"/>
+    <mergeCell ref="F37:I37"/>
+    <mergeCell ref="B69:J69"/>
+    <mergeCell ref="B58:F58"/>
+    <mergeCell ref="G33:I33"/>
+    <mergeCell ref="B35:N35"/>
     <mergeCell ref="B4:N4"/>
     <mergeCell ref="B7:N7"/>
-    <mergeCell ref="B83:J83"/>
-    <mergeCell ref="C31:D31"/>
     <mergeCell ref="B3:N3"/>
     <mergeCell ref="B6:J6"/>
-    <mergeCell ref="G31:I31"/>
+    <mergeCell ref="G32:I32"/>
+    <mergeCell ref="B87:F87"/>
+    <mergeCell ref="B89:J89"/>
+    <mergeCell ref="B85:J85"/>
     <mergeCell ref="B12:N12"/>
     <mergeCell ref="B11:N11"/>
     <mergeCell ref="B2:N2"/>
     <mergeCell ref="B14:N14"/>
-    <mergeCell ref="F35:I35"/>
+    <mergeCell ref="C32:D32"/>
     <mergeCell ref="B8:N8"/>
+    <mergeCell ref="B46:J46"/>
     <mergeCell ref="B13:N13"/>
-    <mergeCell ref="B85:F85"/>
-    <mergeCell ref="B105:J105"/>
-    <mergeCell ref="B58:J58"/>
+    <mergeCell ref="B31:J31"/>
+    <mergeCell ref="B37:E37"/>
+    <mergeCell ref="B34:N34"/>
     <mergeCell ref="B10:N10"/>
   </mergeCells>
-  <conditionalFormatting sqref="N16:N27">
+  <conditionalFormatting sqref="N16:N29">
     <cfRule type="dataBar" priority="1">
       <dataBar minLength="5" maxLength="90" showValue="1">
         <cfvo type="min"/>
@@ -4515,7 +4638,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E16:E27">
+  <conditionalFormatting sqref="E16:E29">
     <cfRule type="dataBar" priority="2">
       <dataBar minLength="5" maxLength="90" showValue="1">
         <cfvo type="min"/>
@@ -4524,7 +4647,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D37:D41">
+  <conditionalFormatting sqref="D39:D43">
     <cfRule type="dataBar" priority="3">
       <dataBar minLength="5" maxLength="90" showValue="1">
         <cfvo type="min"/>
@@ -4533,7 +4656,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H37:H41">
+  <conditionalFormatting sqref="H39:H43">
     <cfRule type="dataBar" priority="4">
       <dataBar minLength="5" maxLength="90" showValue="1">
         <cfvo type="min"/>
@@ -4542,7 +4665,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D60:D65">
+  <conditionalFormatting sqref="D62:D67">
     <cfRule type="dataBar" priority="5">
       <dataBar minLength="5" maxLength="90" showValue="1">
         <cfvo type="min"/>
@@ -4551,7 +4674,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E60:E65">
+  <conditionalFormatting sqref="E62:E67">
     <cfRule type="dataBar" priority="6">
       <dataBar minLength="5" maxLength="90" showValue="1">
         <cfvo type="min"/>
@@ -4560,7 +4683,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C69:C81">
+  <conditionalFormatting sqref="C71:C83">
     <cfRule type="dataBar" priority="7">
       <dataBar minLength="5" maxLength="90" showValue="1">
         <cfvo type="min"/>
@@ -4569,7 +4692,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J69:J81">
+  <conditionalFormatting sqref="J71:J83">
     <cfRule type="dataBar" priority="8">
       <dataBar minLength="5" maxLength="90" showValue="1">
         <cfvo type="min"/>
@@ -4578,7 +4701,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D89:D103">
+  <conditionalFormatting sqref="D91:D105">
     <cfRule type="dataBar" priority="9">
       <dataBar minLength="5" maxLength="90" showValue="1">
         <cfvo type="min"/>
@@ -4587,7 +4710,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F89:F103">
+  <conditionalFormatting sqref="F91:F105">
     <cfRule type="dataBar" priority="10">
       <dataBar minLength="5" maxLength="90" showValue="1">
         <cfvo type="min"/>
@@ -4677,7 +4800,7 @@
     <row r="12">
       <c r="C12" s="72" t="inlineStr">
         <is>
-          <t>⭐⭐ 南茂 (8150) · 10 大戶</t>
+          <t>⭐⭐ 友達 (2409) · 12 大戶</t>
         </is>
       </c>
     </row>
@@ -4719,7 +4842,7 @@
     <row r="19">
       <c r="C19" s="73" t="inlineStr">
         <is>
-          <t>⭐⭐ 南茂 (8150) · 10 大戶</t>
+          <t>⭐⭐ 友達 (2409) · 12 大戶</t>
         </is>
       </c>
     </row>
@@ -4733,21 +4856,21 @@
     <row r="22">
       <c r="C22" s="73" t="inlineStr">
         <is>
-          <t>半導體業 · 5 檔 (42%)</t>
+          <t>半導體業 · 6 檔 (43%)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="C23" s="73" t="inlineStr">
         <is>
-          <t>光電業 · 4 檔 (33%)</t>
+          <t>光電業 · 4 檔 (29%)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="C24" s="73" t="inlineStr">
         <is>
-          <t>電子零組件業 · 2 檔 (17%)</t>
+          <t>電子零組件業 · 3 檔 (21%)</t>
         </is>
       </c>
     </row>
@@ -4810,7 +4933,7 @@
     <row r="36" ht="22" customHeight="1">
       <c r="C36" s="77" t="inlineStr">
         <is>
-          <t>-83 億 淨買</t>
+          <t>-82 億 淨買</t>
         </is>
       </c>
     </row>
@@ -15393,29 +15516,29 @@
       </c>
       <c r="D190" s="138" t="inlineStr">
         <is>
-          <t>台積電(2330)</t>
+          <t>臻鼎-KY(4958)</t>
         </is>
       </c>
       <c r="E190" s="139" t="n">
-        <v>54</v>
+        <v>117</v>
       </c>
       <c r="F190" s="139" t="n">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G190" s="139" t="n">
-        <v>13780</v>
+        <v>6760</v>
       </c>
       <c r="H190" s="139" t="n">
-        <v>13284</v>
+        <v>2895</v>
       </c>
       <c r="I190" s="139" t="n">
-        <v>496</v>
+        <v>3865</v>
       </c>
       <c r="J190" s="140" t="n">
-        <v>2551.81</v>
+        <v>577.78</v>
       </c>
       <c r="K190" s="140" t="n">
-        <v>2554.6</v>
+        <v>579</v>
       </c>
       <c r="L190" s="232">
         <f>F190*(K190-J190)</f>
@@ -15428,31 +15551,31 @@
       <c r="C191" s="141" t="n"/>
       <c r="D191" s="138" t="inlineStr">
         <is>
-          <t>國巨*(2327)</t>
+          <t>友達(2409)</t>
         </is>
       </c>
       <c r="E191" s="139" t="n">
-        <v>98</v>
+        <v>1175</v>
       </c>
       <c r="F191" s="139" t="n">
-        <v>84</v>
+        <v>729</v>
       </c>
       <c r="G191" s="139" t="n">
-        <v>6124</v>
+        <v>4738</v>
       </c>
       <c r="H191" s="139" t="n">
-        <v>5263</v>
+        <v>2919</v>
       </c>
       <c r="I191" s="139" t="n">
-        <v>861</v>
+        <v>1819</v>
       </c>
       <c r="J191" s="140" t="n">
-        <v>624.85</v>
+        <v>40.33</v>
       </c>
       <c r="K191" s="140" t="n">
-        <v>626.6</v>
-      </c>
-      <c r="L191" s="232">
+        <v>40.04</v>
+      </c>
+      <c r="L191" s="233">
         <f>F191*(K191-J191)</f>
         <v/>
       </c>
@@ -15463,29 +15586,29 @@
       <c r="C192" s="141" t="n"/>
       <c r="D192" s="138" t="inlineStr">
         <is>
-          <t>台半(5425)</t>
+          <t>南亞科(2408)</t>
         </is>
       </c>
       <c r="E192" s="139" t="n">
-        <v>420</v>
+        <v>87</v>
       </c>
       <c r="F192" s="139" t="n">
-        <v>200</v>
+        <v>63</v>
       </c>
       <c r="G192" s="139" t="n">
-        <v>4524</v>
+        <v>4549</v>
       </c>
       <c r="H192" s="139" t="n">
-        <v>2202</v>
+        <v>3310</v>
       </c>
       <c r="I192" s="139" t="n">
-        <v>2322</v>
+        <v>1239</v>
       </c>
       <c r="J192" s="140" t="n">
-        <v>107.7</v>
+        <v>522.91</v>
       </c>
       <c r="K192" s="140" t="n">
-        <v>110.08</v>
+        <v>525.3200000000001</v>
       </c>
       <c r="L192" s="232">
         <f>F192*(K192-J192)</f>
@@ -15498,31 +15621,31 @@
       <c r="C193" s="141" t="n"/>
       <c r="D193" s="138" t="inlineStr">
         <is>
-          <t>光聖(6442)</t>
+          <t>國巨*(2327)</t>
         </is>
       </c>
       <c r="E193" s="139" t="n">
-        <v>26</v>
+        <v>53</v>
       </c>
       <c r="F193" s="139" t="n">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="G193" s="139" t="n">
-        <v>4504</v>
+        <v>3353</v>
       </c>
       <c r="H193" s="139" t="n">
-        <v>1317</v>
+        <v>1936</v>
       </c>
       <c r="I193" s="139" t="n">
-        <v>3187</v>
+        <v>1417</v>
       </c>
       <c r="J193" s="140" t="n">
-        <v>1732.31</v>
+        <v>632.72</v>
       </c>
       <c r="K193" s="140" t="n">
-        <v>1646.75</v>
-      </c>
-      <c r="L193" s="233">
+        <v>645.37</v>
+      </c>
+      <c r="L193" s="232">
         <f>F193*(K193-J193)</f>
         <v/>
       </c>
@@ -15537,27 +15660,27 @@
         </is>
       </c>
       <c r="E194" s="139" t="n">
-        <v>286</v>
+        <v>191</v>
       </c>
       <c r="F194" s="139" t="n">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="G194" s="139" t="n">
-        <v>4441</v>
+        <v>2965</v>
       </c>
       <c r="H194" s="139" t="n">
-        <v>392</v>
+        <v>564</v>
       </c>
       <c r="I194" s="139" t="n">
-        <v>4049</v>
+        <v>2401</v>
       </c>
       <c r="J194" s="140" t="n">
-        <v>155.27</v>
+        <v>155.25</v>
       </c>
       <c r="K194" s="140" t="n">
-        <v>156.96</v>
-      </c>
-      <c r="L194" s="232">
+        <v>152.51</v>
+      </c>
+      <c r="L194" s="233">
         <f>F194*(K194-J194)</f>
         <v/>
       </c>
@@ -15568,29 +15691,29 @@
       <c r="C195" s="141" t="n"/>
       <c r="D195" s="138" t="inlineStr">
         <is>
-          <t>穩懋(3105)</t>
+          <t>貿聯-KY(3665)</t>
         </is>
       </c>
       <c r="E195" s="139" t="n">
-        <v>66</v>
+        <v>12</v>
       </c>
       <c r="F195" s="139" t="n">
-        <v>28</v>
+        <v>9</v>
       </c>
       <c r="G195" s="139" t="n">
-        <v>4063</v>
+        <v>2880</v>
       </c>
       <c r="H195" s="139" t="n">
-        <v>1743</v>
+        <v>2290</v>
       </c>
       <c r="I195" s="139" t="n">
-        <v>2320</v>
+        <v>590</v>
       </c>
       <c r="J195" s="140" t="n">
-        <v>615.67</v>
+        <v>2399.67</v>
       </c>
       <c r="K195" s="140" t="n">
-        <v>622.36</v>
+        <v>2543.89</v>
       </c>
       <c r="L195" s="232">
         <f>F195*(K195-J195)</f>
@@ -15603,29 +15726,29 @@
       <c r="C196" s="141" t="n"/>
       <c r="D196" s="138" t="inlineStr">
         <is>
-          <t>臻鼎-KY(4958)</t>
+          <t>台虹(8039)</t>
         </is>
       </c>
       <c r="E196" s="139" t="n">
-        <v>65</v>
+        <v>94</v>
       </c>
       <c r="F196" s="139" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G196" s="139" t="n">
-        <v>3717</v>
+        <v>2828</v>
       </c>
       <c r="H196" s="139" t="n">
-        <v>2313</v>
+        <v>1177</v>
       </c>
       <c r="I196" s="139" t="n">
-        <v>1404</v>
+        <v>1651</v>
       </c>
       <c r="J196" s="140" t="n">
-        <v>571.86</v>
+        <v>300.87</v>
       </c>
       <c r="K196" s="140" t="n">
-        <v>578.2</v>
+        <v>301.87</v>
       </c>
       <c r="L196" s="232">
         <f>F196*(K196-J196)</f>
@@ -15638,29 +15761,29 @@
       <c r="C197" s="141" t="n"/>
       <c r="D197" s="138" t="inlineStr">
         <is>
-          <t>穎崴(6515)</t>
+          <t>合晶(6182)</t>
         </is>
       </c>
       <c r="E197" s="139" t="n">
-        <v>6</v>
+        <v>184</v>
       </c>
       <c r="F197" s="139" t="n">
-        <v>2</v>
+        <v>162</v>
       </c>
       <c r="G197" s="139" t="n">
-        <v>3692</v>
+        <v>2415</v>
       </c>
       <c r="H197" s="139" t="n">
-        <v>1330</v>
+        <v>2131</v>
       </c>
       <c r="I197" s="139" t="n">
-        <v>2362</v>
+        <v>284</v>
       </c>
       <c r="J197" s="140" t="n">
-        <v>6153.67</v>
+        <v>131.24</v>
       </c>
       <c r="K197" s="140" t="n">
-        <v>6648</v>
+        <v>131.52</v>
       </c>
       <c r="L197" s="232">
         <f>F197*(K197-J197)</f>
@@ -15673,31 +15796,31 @@
       <c r="C198" s="141" t="n"/>
       <c r="D198" s="138" t="inlineStr">
         <is>
-          <t>台光電(2383)</t>
+          <t>華新科(2492)</t>
         </is>
       </c>
       <c r="E198" s="139" t="n">
-        <v>6</v>
+        <v>57</v>
       </c>
       <c r="F198" s="139" t="n">
-        <v>1</v>
+        <v>45</v>
       </c>
       <c r="G198" s="139" t="n">
-        <v>3384</v>
+        <v>2108</v>
       </c>
       <c r="H198" s="139" t="n">
-        <v>801</v>
+        <v>1653</v>
       </c>
       <c r="I198" s="139" t="n">
-        <v>2583</v>
+        <v>455</v>
       </c>
       <c r="J198" s="140" t="n">
-        <v>5639.5</v>
+        <v>369.88</v>
       </c>
       <c r="K198" s="140" t="n">
-        <v>8009</v>
-      </c>
-      <c r="L198" s="232">
+        <v>367.4</v>
+      </c>
+      <c r="L198" s="233">
         <f>F198*(K198-J198)</f>
         <v/>
       </c>
@@ -15708,31 +15831,31 @@
       <c r="C199" s="141" t="n"/>
       <c r="D199" s="138" t="inlineStr">
         <is>
-          <t>聯友金屬-創(7610)</t>
+          <t>力成(6239)</t>
         </is>
       </c>
       <c r="E199" s="139" t="n">
-        <v>17</v>
+        <v>62</v>
       </c>
       <c r="F199" s="139" t="n">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="G199" s="139" t="n">
-        <v>3149</v>
+        <v>1877</v>
       </c>
       <c r="H199" s="139" t="n">
-        <v>1882</v>
+        <v>1174</v>
       </c>
       <c r="I199" s="139" t="n">
-        <v>1267</v>
+        <v>703</v>
       </c>
       <c r="J199" s="140" t="n">
-        <v>1852.24</v>
+        <v>302.71</v>
       </c>
       <c r="K199" s="140" t="n">
-        <v>1882.5</v>
-      </c>
-      <c r="L199" s="232">
+        <v>300.95</v>
+      </c>
+      <c r="L199" s="233">
         <f>F199*(K199-J199)</f>
         <v/>
       </c>
@@ -26255,7 +26378,7 @@
     <row r="485" ht="16.5" customHeight="1">
       <c r="A485" s="205" t="inlineStr">
         <is>
-          <t>ⓘ histock top-buyer 資料 fetched @ 2026-10-05 21:49 | 0/17 success</t>
+          <t>ⓘ histock top-buyer 資料 fetched @ 2026-10-05 22:27 | 0/17 success</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-10-07 04:02
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-10.xlsx
+++ b/data/reports/chip_radar_2026-10.xlsx
@@ -24,7 +24,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="28">
+  <numFmts count="29">
     <numFmt numFmtId="164" formatCode="0%&quot; (13/13 ・昨100/5d100)&quot;"/>
     <numFmt numFmtId="165" formatCode="+0&quot; 億 (昨-42/5d-70)&quot;;-0&quot; 億 (昨-42/5d-70)&quot;;0&quot; 億&quot;"/>
     <numFmt numFmtId="166" formatCode="0&quot; 檔 +11億 &quot;&quot;(昨7/5d12)&quot;"/>
@@ -53,6 +53,7 @@
     <numFmt numFmtId="189" formatCode="+0&quot; 億 (昨-82/5d-72)&quot;;-0&quot; 億 (昨-82/5d-72)&quot;;0&quot; 億&quot;"/>
     <numFmt numFmtId="190" formatCode="0&quot; 檔 +92億 &quot;&quot;(昨14/5d9)&quot;"/>
     <numFmt numFmtId="191" formatCode="0.0%&quot; 市-1136億 &quot;&quot;(昨19/5d19)&quot;"/>
+    <numFmt numFmtId="192" formatCode="0&quot; 檔 +91億 &quot;&quot;(昨14/5d9)&quot;"/>
   </numFmts>
   <fonts count="52">
     <font>
@@ -617,7 +618,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="252">
+  <cellXfs count="253">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1202,6 +1203,9 @@
     <xf numFmtId="191" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="192" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1310,15 +1314,15 @@
 真共識訊號被稀釋.</t>
       </text>
     </comment>
-    <comment ref="D24" authorId="0" shapeId="0">
+    <comment ref="D25" authorId="0" shapeId="0">
       <text>
         <t>⚠️ 假共識警示
-領頭大戶「陳族元」獨佔比 74.6%
-  • 領頭金額 13,621 萬
-  • 合計淨買 18,270 萬
+領頭大戶「陳族元」獨佔比 64.7%
+  • 領頭金額 8,526 萬
+  • 合計淨買 13,174 萬
   • 大戶數 10 位 (名義共識)
 判讀: 名義 10 位大戶共識,
-實質 1 人下注佔 75%,
+實質 1 人下注佔 65%,
 剩餘 9 位為陪襯小單,
 真共識訊號被稀釋.</t>
       </text>
@@ -1979,7 +1983,7 @@
         <v>13</v>
       </c>
       <c r="F19" s="15" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G19" s="16" t="inlineStr">
         <is>
@@ -1987,7 +1991,7 @@
         </is>
       </c>
       <c r="H19" s="17" t="n">
-        <v>21768</v>
+        <v>20853</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -2009,7 +2013,7 @@
         <v>10</v>
       </c>
       <c r="N19" s="17" t="n">
-        <v>87454</v>
+        <v>86539</v>
       </c>
     </row>
     <row r="20">
@@ -2222,49 +2226,49 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>1709</t>
-        </is>
-      </c>
-      <c r="D24" s="21" t="inlineStr">
-        <is>
-          <t>📌 ⚠️ 和益</t>
+          <t>4979</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>華星光</t>
         </is>
       </c>
       <c r="E24" s="14" t="n">
         <v>10</v>
       </c>
       <c r="F24" s="15" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="G24" s="16" t="inlineStr">
         <is>
-          <t>陳族元</t>
+          <t>陳律師</t>
         </is>
       </c>
       <c r="H24" s="17" t="n">
-        <v>13622</v>
+        <v>8355</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>強森</t>
+          <t>張濬安</t>
         </is>
       </c>
       <c r="J24" s="18" t="n">
-        <v>1333</v>
+        <v>1484</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>張濬安</t>
+          <t>林滄海</t>
         </is>
       </c>
       <c r="L24" s="18" t="n">
-        <v>735</v>
+        <v>1251</v>
       </c>
       <c r="M24" s="19" t="n">
         <v>7</v>
       </c>
       <c r="N24" s="17" t="n">
-        <v>18270</v>
+        <v>16974</v>
       </c>
     </row>
     <row r="25">
@@ -2273,49 +2277,49 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>4979</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>華星光</t>
+          <t>1709</t>
+        </is>
+      </c>
+      <c r="D25" s="21" t="inlineStr">
+        <is>
+          <t>📌 ⚠️ 和益</t>
         </is>
       </c>
       <c r="E25" s="14" t="n">
         <v>10</v>
       </c>
       <c r="F25" s="15" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="G25" s="16" t="inlineStr">
         <is>
-          <t>陳律師</t>
+          <t>陳族元</t>
         </is>
       </c>
       <c r="H25" s="17" t="n">
-        <v>8355</v>
+        <v>8526</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
+          <t>強森</t>
+        </is>
+      </c>
+      <c r="J25" s="18" t="n">
+        <v>1333</v>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
           <t>張濬安</t>
         </is>
       </c>
-      <c r="J25" s="18" t="n">
-        <v>1484</v>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>林滄海</t>
-        </is>
-      </c>
       <c r="L25" s="18" t="n">
-        <v>1251</v>
+        <v>735</v>
       </c>
       <c r="M25" s="19" t="n">
         <v>7</v>
       </c>
       <c r="N25" s="17" t="n">
-        <v>16974</v>
+        <v>13174</v>
       </c>
     </row>
     <row r="26">
@@ -2387,23 +2391,23 @@
         <v>11</v>
       </c>
       <c r="F27" s="15" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G27" s="16" t="inlineStr">
         <is>
+          <t>林滄海</t>
+        </is>
+      </c>
+      <c r="H27" s="17" t="n">
+        <v>424</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
           <t>陳族元</t>
         </is>
       </c>
-      <c r="H27" s="17" t="n">
-        <v>450</v>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>林滄海</t>
-        </is>
-      </c>
       <c r="J27" s="18" t="n">
-        <v>424</v>
+        <v>390</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>
@@ -2417,7 +2421,7 @@
         <v>8</v>
       </c>
       <c r="N27" s="17" t="n">
-        <v>2248</v>
+        <v>2187</v>
       </c>
     </row>
     <row r="29" ht="22" customHeight="1">
@@ -2442,7 +2446,7 @@
         </is>
       </c>
       <c r="G30" s="249" t="n">
-        <v>-154.55198</v>
+        <v>-154.10581</v>
       </c>
     </row>
     <row r="31" ht="28" customHeight="1">
@@ -2451,7 +2455,7 @@
           <t>Q3 強共識股</t>
         </is>
       </c>
-      <c r="C31" s="250" t="n">
+      <c r="C31" s="252" t="n">
         <v>12</v>
       </c>
       <c r="F31" s="23" t="inlineStr">
@@ -2460,7 +2464,7 @@
         </is>
       </c>
       <c r="G31" s="251" t="n">
-        <v>0.1914306394596117</v>
+        <v>0.1911346159181977</v>
       </c>
     </row>
     <row r="32" ht="22" customHeight="1">
@@ -2543,7 +2547,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>30.5%</t>
+          <t>30.6%</t>
         </is>
       </c>
       <c r="F37" t="n">
@@ -2571,11 +2575,11 @@
         </is>
       </c>
       <c r="D38" s="34" t="n">
-        <v>1191366</v>
+        <v>1178781</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>23.2%</t>
+          <t>23.0%</t>
         </is>
       </c>
       <c r="F38" t="n">
@@ -2785,7 +2789,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>陳族元</t>
+          <t>Tradow</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2795,12 +2799,12 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>陳族元 今日買進 9 檔新標的 (過去從沒買過)</t>
+          <t>Tradow 今日買進 8 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>9 檔</t>
+          <t>8 檔</t>
         </is>
       </c>
     </row>
@@ -2812,7 +2816,7 @@
       </c>
       <c r="C49" s="41" t="inlineStr">
         <is>
-          <t>Tradow</t>
+          <t>強森</t>
         </is>
       </c>
       <c r="D49" s="41" t="inlineStr">
@@ -2822,12 +2826,12 @@
       </c>
       <c r="E49" s="41" t="inlineStr">
         <is>
-          <t>Tradow 今日買進 8 檔新標的 (過去從沒買過)</t>
+          <t>強森 今日買進 7 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F49" s="41" t="inlineStr">
         <is>
-          <t>8 檔</t>
+          <t>7 檔</t>
         </is>
       </c>
     </row>
@@ -2839,7 +2843,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>強森</t>
+          <t>迷你哥/松山哥</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -2849,12 +2853,12 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>強森 今日買進 7 檔新標的 (過去從沒買過)</t>
+          <t>迷你哥/松山哥 今日買進 6 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>7 檔</t>
+          <t>6 檔</t>
         </is>
       </c>
     </row>
@@ -2866,7 +2870,7 @@
       </c>
       <c r="C51" s="41" t="inlineStr">
         <is>
-          <t>迷你哥/松山哥</t>
+          <t>陳律師</t>
         </is>
       </c>
       <c r="D51" s="41" t="inlineStr">
@@ -2876,7 +2880,7 @@
       </c>
       <c r="E51" s="41" t="inlineStr">
         <is>
-          <t>迷你哥/松山哥 今日買進 6 檔新標的 (過去從沒買過)</t>
+          <t>陳律師 今日買進 6 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F51" s="41" t="inlineStr">
@@ -2893,7 +2897,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>陳律師</t>
+          <t>陳族元</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2903,7 +2907,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>陳律師 今日買進 6 檔新標的 (過去從沒買過)</t>
+          <t>陳族元 今日買進 6 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -3274,7 +3278,7 @@
         </is>
       </c>
       <c r="C70" s="34" t="n">
-        <v>1115287</v>
+        <v>1101644</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -3282,7 +3286,7 @@
         </is>
       </c>
       <c r="E70" s="34" t="n">
-        <v>110929</v>
+        <v>108141</v>
       </c>
       <c r="F70" t="inlineStr">
         <is>
@@ -3301,7 +3305,7 @@
         <v>61976</v>
       </c>
       <c r="J70" s="213" t="n">
-        <v>0.2178465389279929</v>
+        <v>0.218013836226448</v>
       </c>
     </row>
     <row r="71">
@@ -4804,7 +4808,7 @@
     <row r="29" ht="22" customHeight="1">
       <c r="C29" s="77" t="inlineStr">
         <is>
-          <t>-155 億 淨買</t>
+          <t>-154 億 淨買</t>
         </is>
       </c>
     </row>
@@ -15774,10 +15778,10 @@
         </is>
       </c>
       <c r="E190" s="139" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F190" s="139" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G190" s="139" t="n">
         <v>11559</v>
@@ -15789,12 +15793,12 @@
         <v>9717</v>
       </c>
       <c r="J190" s="140" t="n">
-        <v>1751.33</v>
+        <v>1725.19</v>
       </c>
       <c r="K190" s="140" t="n">
-        <v>1842.2</v>
-      </c>
-      <c r="L190" s="232">
+        <v>1674.73</v>
+      </c>
+      <c r="L190" s="233">
         <f>F190*(K190-J190)</f>
         <v/>
       </c>
@@ -15809,10 +15813,10 @@
         </is>
       </c>
       <c r="E191" s="139" t="n">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="F191" s="139" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G191" s="139" t="n">
         <v>9693</v>
@@ -15824,12 +15828,12 @@
         <v>9086</v>
       </c>
       <c r="J191" s="140" t="n">
-        <v>255.74</v>
+        <v>257.1</v>
       </c>
       <c r="K191" s="140" t="n">
-        <v>253.04</v>
-      </c>
-      <c r="L191" s="233">
+        <v>264.04</v>
+      </c>
+      <c r="L191" s="232">
         <f>F191*(K191-J191)</f>
         <v/>
       </c>
@@ -15840,29 +15844,29 @@
       <c r="C192" s="141" t="n"/>
       <c r="D192" s="138" t="inlineStr">
         <is>
-          <t>和益(1709)</t>
+          <t>信驊(5274)</t>
         </is>
       </c>
       <c r="E192" s="139" t="n">
-        <v>1085</v>
+        <v>3</v>
       </c>
       <c r="F192" s="139" t="n">
-        <v>280</v>
+        <v>0</v>
       </c>
       <c r="G192" s="139" t="n">
-        <v>6868</v>
+        <v>5851</v>
       </c>
       <c r="H192" s="139" t="n">
-        <v>1772</v>
+        <v>0</v>
       </c>
       <c r="I192" s="139" t="n">
-        <v>5096</v>
+        <v>5851</v>
       </c>
       <c r="J192" s="140" t="n">
-        <v>63.3</v>
+        <v>19502.33</v>
       </c>
       <c r="K192" s="140" t="n">
-        <v>63.3</v>
+        <v>0</v>
       </c>
       <c r="L192" s="232">
         <f>F192*(K192-J192)</f>
@@ -15875,29 +15879,29 @@
       <c r="C193" s="141" t="n"/>
       <c r="D193" s="138" t="inlineStr">
         <is>
-          <t>信驊(5274)</t>
+          <t>聯發科(2454)</t>
         </is>
       </c>
       <c r="E193" s="139" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="F193" s="139" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G193" s="139" t="n">
-        <v>5851</v>
+        <v>5057</v>
       </c>
       <c r="H193" s="139" t="n">
-        <v>0</v>
+        <v>1170</v>
       </c>
       <c r="I193" s="139" t="n">
-        <v>5851</v>
+        <v>3887</v>
       </c>
       <c r="J193" s="140" t="n">
-        <v>19502.33</v>
+        <v>5057.2</v>
       </c>
       <c r="K193" s="140" t="n">
-        <v>0</v>
+        <v>5847.5</v>
       </c>
       <c r="L193" s="232">
         <f>F193*(K193-J193)</f>
@@ -15910,31 +15914,31 @@
       <c r="C194" s="141" t="n"/>
       <c r="D194" s="138" t="inlineStr">
         <is>
-          <t>聯發科(2454)</t>
+          <t>金居(8358)</t>
         </is>
       </c>
       <c r="E194" s="139" t="n">
-        <v>10</v>
+        <v>81</v>
       </c>
       <c r="F194" s="139" t="n">
-        <v>2</v>
+        <v>39</v>
       </c>
       <c r="G194" s="139" t="n">
-        <v>5057</v>
+        <v>4485</v>
       </c>
       <c r="H194" s="139" t="n">
-        <v>1170</v>
+        <v>2133</v>
       </c>
       <c r="I194" s="139" t="n">
-        <v>3887</v>
+        <v>2352</v>
       </c>
       <c r="J194" s="140" t="n">
-        <v>5057.2</v>
+        <v>553.67</v>
       </c>
       <c r="K194" s="140" t="n">
-        <v>5847.5</v>
-      </c>
-      <c r="L194" s="232">
+        <v>546.85</v>
+      </c>
+      <c r="L194" s="233">
         <f>F194*(K194-J194)</f>
         <v/>
       </c>
@@ -15945,29 +15949,29 @@
       <c r="C195" s="141" t="n"/>
       <c r="D195" s="138" t="inlineStr">
         <is>
-          <t>金居(8358)</t>
+          <t>華通(2313)</t>
         </is>
       </c>
       <c r="E195" s="139" t="n">
-        <v>81</v>
+        <v>178</v>
       </c>
       <c r="F195" s="139" t="n">
-        <v>39</v>
+        <v>139</v>
       </c>
       <c r="G195" s="139" t="n">
-        <v>4485</v>
+        <v>4484</v>
       </c>
       <c r="H195" s="139" t="n">
-        <v>2133</v>
+        <v>3493</v>
       </c>
       <c r="I195" s="139" t="n">
-        <v>2352</v>
+        <v>991</v>
       </c>
       <c r="J195" s="140" t="n">
-        <v>553.67</v>
+        <v>251.9</v>
       </c>
       <c r="K195" s="140" t="n">
-        <v>546.85</v>
+        <v>251.27</v>
       </c>
       <c r="L195" s="233">
         <f>F195*(K195-J195)</f>
@@ -15980,29 +15984,29 @@
       <c r="C196" s="141" t="n"/>
       <c r="D196" s="138" t="inlineStr">
         <is>
-          <t>華通(2313)</t>
+          <t>台積電(2330)</t>
         </is>
       </c>
       <c r="E196" s="139" t="n">
-        <v>178</v>
+        <v>15</v>
       </c>
       <c r="F196" s="139" t="n">
-        <v>139</v>
+        <v>4</v>
       </c>
       <c r="G196" s="139" t="n">
-        <v>4484</v>
+        <v>3997</v>
       </c>
       <c r="H196" s="139" t="n">
-        <v>3493</v>
+        <v>966</v>
       </c>
       <c r="I196" s="139" t="n">
-        <v>991</v>
+        <v>3031</v>
       </c>
       <c r="J196" s="140" t="n">
-        <v>251.9</v>
+        <v>2664.6</v>
       </c>
       <c r="K196" s="140" t="n">
-        <v>251.27</v>
+        <v>2416</v>
       </c>
       <c r="L196" s="233">
         <f>F196*(K196-J196)</f>
@@ -16015,29 +16019,29 @@
       <c r="C197" s="141" t="n"/>
       <c r="D197" s="138" t="inlineStr">
         <is>
-          <t>台積電(2330)</t>
+          <t>南亞(1303)</t>
         </is>
       </c>
       <c r="E197" s="139" t="n">
-        <v>15</v>
+        <v>117</v>
       </c>
       <c r="F197" s="139" t="n">
-        <v>4</v>
+        <v>37</v>
       </c>
       <c r="G197" s="139" t="n">
-        <v>3997</v>
+        <v>3388</v>
       </c>
       <c r="H197" s="139" t="n">
-        <v>966</v>
+        <v>1062</v>
       </c>
       <c r="I197" s="139" t="n">
-        <v>3031</v>
+        <v>2326</v>
       </c>
       <c r="J197" s="140" t="n">
-        <v>2664.6</v>
+        <v>289.57</v>
       </c>
       <c r="K197" s="140" t="n">
-        <v>2416</v>
+        <v>286.95</v>
       </c>
       <c r="L197" s="233">
         <f>F197*(K197-J197)</f>
@@ -16050,29 +16054,29 @@
       <c r="C198" s="141" t="n"/>
       <c r="D198" s="138" t="inlineStr">
         <is>
-          <t>南亞(1303)</t>
+          <t>國巨*(2327)</t>
         </is>
       </c>
       <c r="E198" s="139" t="n">
-        <v>116</v>
+        <v>51</v>
       </c>
       <c r="F198" s="139" t="n">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="G198" s="139" t="n">
-        <v>3388</v>
+        <v>3156</v>
       </c>
       <c r="H198" s="139" t="n">
-        <v>1062</v>
+        <v>1638</v>
       </c>
       <c r="I198" s="139" t="n">
-        <v>2326</v>
+        <v>1518</v>
       </c>
       <c r="J198" s="140" t="n">
-        <v>292.07</v>
+        <v>618.92</v>
       </c>
       <c r="K198" s="140" t="n">
-        <v>294.92</v>
+        <v>629.85</v>
       </c>
       <c r="L198" s="232">
         <f>F198*(K198-J198)</f>
@@ -16085,29 +16089,29 @@
       <c r="C199" s="141" t="n"/>
       <c r="D199" s="138" t="inlineStr">
         <is>
-          <t>國巨*(2327)</t>
+          <t>晶心科(6533)</t>
         </is>
       </c>
       <c r="E199" s="139" t="n">
-        <v>51</v>
+        <v>85</v>
       </c>
       <c r="F199" s="139" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="G199" s="139" t="n">
-        <v>3156</v>
+        <v>2936</v>
       </c>
       <c r="H199" s="139" t="n">
-        <v>1638</v>
+        <v>0</v>
       </c>
       <c r="I199" s="139" t="n">
-        <v>1518</v>
+        <v>2936</v>
       </c>
       <c r="J199" s="140" t="n">
-        <v>618.92</v>
+        <v>345.39</v>
       </c>
       <c r="K199" s="140" t="n">
-        <v>629.85</v>
+        <v>0</v>
       </c>
       <c r="L199" s="232">
         <f>F199*(K199-J199)</f>
@@ -26426,7 +26430,7 @@
     <row r="485" ht="16.5" customHeight="1">
       <c r="A485" s="205" t="inlineStr">
         <is>
-          <t>ⓘ histock top-buyer 資料 fetched @ 2026-10-06 19:10 | 0/5 success</t>
+          <t>ⓘ histock top-buyer 資料 fetched @ 2026-10-06 20:02 | 0/5 success</t>
         </is>
       </c>
     </row>

</xml_diff>